<commit_message>
HP: drop Bundle Detail price to sentinel; harden parser + currency labels
- Bundle Detail rows now carry cost=0 (the price lives on the Bundle
  parent); AnzGenericWriter emits the 0.000001 sentinel on the local
  Cost column. This also corrects the computed total (no double-count).
- Harden HpBidXlsxParser: blank qty/min cells default to 0 instead of
  throwing; Bundle Detail sub-sequencing anchors to the most recent
  Bundle parent rather than any preceding Part Number.
- Add X-Currency response header (AUD for HP, USD for Nutanix); the
  success toast and ValidationWarningModal now label totals with it
  instead of a hard-coded USD.
- Extract CRM template names to frontend src/constants.ts (no more
  magic 'Uplift' string).
- Regenerate the 4 HP golden workbooks; update parser/API test
  assertions (X-Currency, Bundle Detail cost, computed total). 129 tests pass.
- Update AGENTS.md, docs/hp_bid_xlsx.md, docs/output_mapping.md;
  remove the completed hp_bid_plan.md handoff doc.
</commit_message>
<xml_diff>
--- a/samples/outputs/Deals20260518T034809_HPI_NoCalculation_parsed.xlsx
+++ b/samples/outputs/Deals20260518T034809_HPI_NoCalculation_parsed.xlsx
@@ -2778,7 +2778,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="I7" s="0">
-        <x:v>713.26</x:v>
+        <x:v>1E-06</x:v>
       </x:c>
       <x:c r="W7" s="0">
         <x:v>1</x:v>
@@ -2801,7 +2801,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="I8" s="0">
-        <x:v>0.03</x:v>
+        <x:v>1E-06</x:v>
       </x:c>
       <x:c r="W8" s="0">
         <x:v>1</x:v>
@@ -2824,7 +2824,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="I9" s="0">
-        <x:v>0.03</x:v>
+        <x:v>1E-06</x:v>
       </x:c>
       <x:c r="W9" s="0">
         <x:v>1</x:v>
@@ -2847,7 +2847,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="I10" s="0">
-        <x:v>319.35</x:v>
+        <x:v>1E-06</x:v>
       </x:c>
       <x:c r="W10" s="0">
         <x:v>1</x:v>
@@ -2870,7 +2870,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="I11" s="0">
-        <x:v>0.03</x:v>
+        <x:v>1E-06</x:v>
       </x:c>
       <x:c r="W11" s="0">
         <x:v>1</x:v>
@@ -2893,7 +2893,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="I12" s="0">
-        <x:v>0</x:v>
+        <x:v>1E-06</x:v>
       </x:c>
       <x:c r="W12" s="0">
         <x:v>1</x:v>
@@ -2916,7 +2916,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="I13" s="0">
-        <x:v>30.8</x:v>
+        <x:v>1E-06</x:v>
       </x:c>
       <x:c r="W13" s="0">
         <x:v>1</x:v>
@@ -2939,7 +2939,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="I14" s="0">
-        <x:v>157.19</x:v>
+        <x:v>1E-06</x:v>
       </x:c>
       <x:c r="W14" s="0">
         <x:v>1</x:v>
@@ -2962,7 +2962,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="I15" s="0">
-        <x:v>534.96</x:v>
+        <x:v>1E-06</x:v>
       </x:c>
       <x:c r="W15" s="0">
         <x:v>1</x:v>
@@ -2985,7 +2985,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="I16" s="0">
-        <x:v>440</x:v>
+        <x:v>1E-06</x:v>
       </x:c>
       <x:c r="W16" s="0">
         <x:v>1</x:v>
@@ -3008,7 +3008,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="I17" s="0">
-        <x:v>0.03</x:v>
+        <x:v>1E-06</x:v>
       </x:c>
       <x:c r="W17" s="0">
         <x:v>1</x:v>
@@ -3031,7 +3031,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="I18" s="0">
-        <x:v>15.52</x:v>
+        <x:v>1E-06</x:v>
       </x:c>
       <x:c r="W18" s="0">
         <x:v>1</x:v>
@@ -3054,7 +3054,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="I19" s="0">
-        <x:v>19.14</x:v>
+        <x:v>1E-06</x:v>
       </x:c>
       <x:c r="W19" s="0">
         <x:v>1</x:v>
@@ -3077,7 +3077,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="I20" s="0">
-        <x:v>0.05</x:v>
+        <x:v>1E-06</x:v>
       </x:c>
       <x:c r="W20" s="0">
         <x:v>1</x:v>
@@ -3100,7 +3100,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="I21" s="0">
-        <x:v>1.73</x:v>
+        <x:v>1E-06</x:v>
       </x:c>
       <x:c r="W21" s="0">
         <x:v>1</x:v>
@@ -3123,7 +3123,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="I22" s="0">
-        <x:v>0.03</x:v>
+        <x:v>1E-06</x:v>
       </x:c>
       <x:c r="W22" s="0">
         <x:v>1</x:v>
@@ -3146,7 +3146,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="I23" s="0">
-        <x:v>54.17</x:v>
+        <x:v>1E-06</x:v>
       </x:c>
       <x:c r="W23" s="0">
         <x:v>1</x:v>
@@ -3169,7 +3169,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="I24" s="0">
-        <x:v>22.27</x:v>
+        <x:v>1E-06</x:v>
       </x:c>
       <x:c r="W24" s="0">
         <x:v>1</x:v>
@@ -3192,7 +3192,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="I25" s="0">
-        <x:v>39.26</x:v>
+        <x:v>1E-06</x:v>
       </x:c>
       <x:c r="W25" s="0">
         <x:v>1</x:v>
@@ -3215,7 +3215,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="I26" s="0">
-        <x:v>0</x:v>
+        <x:v>1E-06</x:v>
       </x:c>
       <x:c r="W26" s="0">
         <x:v>1</x:v>
@@ -3238,7 +3238,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="I27" s="0">
-        <x:v>1.1</x:v>
+        <x:v>1E-06</x:v>
       </x:c>
       <x:c r="W27" s="0">
         <x:v>1</x:v>
@@ -3261,7 +3261,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="I28" s="0">
-        <x:v>0</x:v>
+        <x:v>1E-06</x:v>
       </x:c>
       <x:c r="W28" s="0">
         <x:v>1</x:v>
@@ -3284,7 +3284,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="I29" s="0">
-        <x:v>2.03</x:v>
+        <x:v>1E-06</x:v>
       </x:c>
       <x:c r="W29" s="0">
         <x:v>1</x:v>
@@ -3307,7 +3307,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="I30" s="0">
-        <x:v>0</x:v>
+        <x:v>1E-06</x:v>
       </x:c>
       <x:c r="W30" s="0">
         <x:v>1</x:v>
@@ -3330,7 +3330,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="I31" s="0">
-        <x:v>33.47</x:v>
+        <x:v>1E-06</x:v>
       </x:c>
       <x:c r="W31" s="0">
         <x:v>1</x:v>
@@ -3353,7 +3353,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="I32" s="0">
-        <x:v>0</x:v>
+        <x:v>1E-06</x:v>
       </x:c>
       <x:c r="W32" s="0">
         <x:v>1</x:v>
@@ -3376,7 +3376,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="I33" s="0">
-        <x:v>0.03</x:v>
+        <x:v>1E-06</x:v>
       </x:c>
       <x:c r="W33" s="0">
         <x:v>1</x:v>
@@ -3399,7 +3399,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="I34" s="0">
-        <x:v>0.03</x:v>
+        <x:v>1E-06</x:v>
       </x:c>
       <x:c r="W34" s="0">
         <x:v>1</x:v>
@@ -3422,7 +3422,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="I35" s="0">
-        <x:v>2.63</x:v>
+        <x:v>1E-06</x:v>
       </x:c>
       <x:c r="W35" s="0">
         <x:v>1</x:v>
@@ -3445,7 +3445,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="I36" s="0">
-        <x:v>0.03</x:v>
+        <x:v>1E-06</x:v>
       </x:c>
       <x:c r="W36" s="0">
         <x:v>1</x:v>
@@ -3468,7 +3468,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="I37" s="0">
-        <x:v>0.03</x:v>
+        <x:v>1E-06</x:v>
       </x:c>
       <x:c r="W37" s="0">
         <x:v>1</x:v>
@@ -3491,7 +3491,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="I38" s="0">
-        <x:v>0.03</x:v>
+        <x:v>1E-06</x:v>
       </x:c>
       <x:c r="W38" s="0">
         <x:v>1</x:v>
@@ -3514,7 +3514,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="I39" s="0">
-        <x:v>0.71</x:v>
+        <x:v>1E-06</x:v>
       </x:c>
       <x:c r="W39" s="0">
         <x:v>1</x:v>
@@ -3560,7 +3560,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="I41" s="0">
-        <x:v>869.6</x:v>
+        <x:v>1E-06</x:v>
       </x:c>
       <x:c r="W41" s="0">
         <x:v>1</x:v>
@@ -3583,7 +3583,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="I42" s="0">
-        <x:v>0.03</x:v>
+        <x:v>1E-06</x:v>
       </x:c>
       <x:c r="W42" s="0">
         <x:v>1</x:v>
@@ -3606,7 +3606,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="I43" s="0">
-        <x:v>0.03</x:v>
+        <x:v>1E-06</x:v>
       </x:c>
       <x:c r="W43" s="0">
         <x:v>1</x:v>
@@ -3629,7 +3629,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="I44" s="0">
-        <x:v>285.7</x:v>
+        <x:v>1E-06</x:v>
       </x:c>
       <x:c r="W44" s="0">
         <x:v>1</x:v>
@@ -3652,7 +3652,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="I45" s="0">
-        <x:v>0.03</x:v>
+        <x:v>1E-06</x:v>
       </x:c>
       <x:c r="W45" s="0">
         <x:v>1</x:v>
@@ -3675,7 +3675,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="I46" s="0">
-        <x:v>0</x:v>
+        <x:v>1E-06</x:v>
       </x:c>
       <x:c r="W46" s="0">
         <x:v>1</x:v>
@@ -3698,7 +3698,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="I47" s="0">
-        <x:v>30.8</x:v>
+        <x:v>1E-06</x:v>
       </x:c>
       <x:c r="W47" s="0">
         <x:v>1</x:v>
@@ -3721,7 +3721,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="I48" s="0">
-        <x:v>126.36</x:v>
+        <x:v>1E-06</x:v>
       </x:c>
       <x:c r="W48" s="0">
         <x:v>1</x:v>
@@ -3744,7 +3744,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="I49" s="0">
-        <x:v>1069.92</x:v>
+        <x:v>1E-06</x:v>
       </x:c>
       <x:c r="W49" s="0">
         <x:v>1</x:v>
@@ -3767,7 +3767,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="I50" s="0">
-        <x:v>440</x:v>
+        <x:v>1E-06</x:v>
       </x:c>
       <x:c r="W50" s="0">
         <x:v>1</x:v>
@@ -3790,7 +3790,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="I51" s="0">
-        <x:v>0.03</x:v>
+        <x:v>1E-06</x:v>
       </x:c>
       <x:c r="W51" s="0">
         <x:v>1</x:v>
@@ -3813,7 +3813,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="I52" s="0">
-        <x:v>15.52</x:v>
+        <x:v>1E-06</x:v>
       </x:c>
       <x:c r="W52" s="0">
         <x:v>1</x:v>
@@ -3836,7 +3836,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="I53" s="0">
-        <x:v>19.14</x:v>
+        <x:v>1E-06</x:v>
       </x:c>
       <x:c r="W53" s="0">
         <x:v>1</x:v>
@@ -3859,7 +3859,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="I54" s="0">
-        <x:v>0.05</x:v>
+        <x:v>1E-06</x:v>
       </x:c>
       <x:c r="W54" s="0">
         <x:v>1</x:v>
@@ -3882,7 +3882,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="I55" s="0">
-        <x:v>1.73</x:v>
+        <x:v>1E-06</x:v>
       </x:c>
       <x:c r="W55" s="0">
         <x:v>1</x:v>
@@ -3905,7 +3905,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="I56" s="0">
-        <x:v>0.03</x:v>
+        <x:v>1E-06</x:v>
       </x:c>
       <x:c r="W56" s="0">
         <x:v>1</x:v>
@@ -3928,7 +3928,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="I57" s="0">
-        <x:v>53.61</x:v>
+        <x:v>1E-06</x:v>
       </x:c>
       <x:c r="W57" s="0">
         <x:v>1</x:v>
@@ -3951,7 +3951,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="I58" s="0">
-        <x:v>22.27</x:v>
+        <x:v>1E-06</x:v>
       </x:c>
       <x:c r="W58" s="0">
         <x:v>1</x:v>
@@ -3974,7 +3974,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="I59" s="0">
-        <x:v>39.26</x:v>
+        <x:v>1E-06</x:v>
       </x:c>
       <x:c r="W59" s="0">
         <x:v>1</x:v>
@@ -3997,7 +3997,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="I60" s="0">
-        <x:v>0</x:v>
+        <x:v>1E-06</x:v>
       </x:c>
       <x:c r="W60" s="0">
         <x:v>1</x:v>
@@ -4020,7 +4020,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="I61" s="0">
-        <x:v>1.1</x:v>
+        <x:v>1E-06</x:v>
       </x:c>
       <x:c r="W61" s="0">
         <x:v>1</x:v>
@@ -4043,7 +4043,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="I62" s="0">
-        <x:v>0</x:v>
+        <x:v>1E-06</x:v>
       </x:c>
       <x:c r="W62" s="0">
         <x:v>1</x:v>
@@ -4066,7 +4066,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="I63" s="0">
-        <x:v>2.03</x:v>
+        <x:v>1E-06</x:v>
       </x:c>
       <x:c r="W63" s="0">
         <x:v>1</x:v>
@@ -4089,7 +4089,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="I64" s="0">
-        <x:v>0</x:v>
+        <x:v>1E-06</x:v>
       </x:c>
       <x:c r="W64" s="0">
         <x:v>1</x:v>
@@ -4112,7 +4112,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="I65" s="0">
-        <x:v>33.47</x:v>
+        <x:v>1E-06</x:v>
       </x:c>
       <x:c r="W65" s="0">
         <x:v>1</x:v>
@@ -4135,7 +4135,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="I66" s="0">
-        <x:v>0</x:v>
+        <x:v>1E-06</x:v>
       </x:c>
       <x:c r="W66" s="0">
         <x:v>1</x:v>
@@ -4158,7 +4158,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="I67" s="0">
-        <x:v>0.03</x:v>
+        <x:v>1E-06</x:v>
       </x:c>
       <x:c r="W67" s="0">
         <x:v>1</x:v>
@@ -4181,7 +4181,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="I68" s="0">
-        <x:v>0.03</x:v>
+        <x:v>1E-06</x:v>
       </x:c>
       <x:c r="W68" s="0">
         <x:v>1</x:v>
@@ -4204,7 +4204,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="I69" s="0">
-        <x:v>2.63</x:v>
+        <x:v>1E-06</x:v>
       </x:c>
       <x:c r="W69" s="0">
         <x:v>1</x:v>
@@ -4227,7 +4227,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="I70" s="0">
-        <x:v>0.03</x:v>
+        <x:v>1E-06</x:v>
       </x:c>
       <x:c r="W70" s="0">
         <x:v>1</x:v>
@@ -4250,7 +4250,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="I71" s="0">
-        <x:v>0.03</x:v>
+        <x:v>1E-06</x:v>
       </x:c>
       <x:c r="W71" s="0">
         <x:v>1</x:v>
@@ -4273,7 +4273,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="I72" s="0">
-        <x:v>0.03</x:v>
+        <x:v>1E-06</x:v>
       </x:c>
       <x:c r="W72" s="0">
         <x:v>1</x:v>
@@ -4296,7 +4296,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="I73" s="0">
-        <x:v>0.71</x:v>
+        <x:v>1E-06</x:v>
       </x:c>
       <x:c r="W73" s="0">
         <x:v>1</x:v>
@@ -4342,7 +4342,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="I75" s="0">
-        <x:v>604.35</x:v>
+        <x:v>1E-06</x:v>
       </x:c>
       <x:c r="W75" s="0">
         <x:v>1</x:v>
@@ -4365,7 +4365,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="I76" s="0">
-        <x:v>0.03</x:v>
+        <x:v>1E-06</x:v>
       </x:c>
       <x:c r="W76" s="0">
         <x:v>1</x:v>
@@ -4388,7 +4388,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="I77" s="0">
-        <x:v>0.03</x:v>
+        <x:v>1E-06</x:v>
       </x:c>
       <x:c r="W77" s="0">
         <x:v>1</x:v>
@@ -4411,7 +4411,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="I78" s="0">
-        <x:v>271.59</x:v>
+        <x:v>1E-06</x:v>
       </x:c>
       <x:c r="W78" s="0">
         <x:v>1</x:v>
@@ -4434,7 +4434,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="I79" s="0">
-        <x:v>0.03</x:v>
+        <x:v>1E-06</x:v>
       </x:c>
       <x:c r="W79" s="0">
         <x:v>1</x:v>
@@ -4457,7 +4457,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="I80" s="0">
-        <x:v>0</x:v>
+        <x:v>1E-06</x:v>
       </x:c>
       <x:c r="W80" s="0">
         <x:v>1</x:v>
@@ -4480,7 +4480,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="I81" s="0">
-        <x:v>30.8</x:v>
+        <x:v>1E-06</x:v>
       </x:c>
       <x:c r="W81" s="0">
         <x:v>1</x:v>
@@ -4503,7 +4503,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="I82" s="0">
-        <x:v>154</x:v>
+        <x:v>1E-06</x:v>
       </x:c>
       <x:c r="W82" s="0">
         <x:v>1</x:v>
@@ -4526,7 +4526,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="I83" s="0">
-        <x:v>534.96</x:v>
+        <x:v>1E-06</x:v>
       </x:c>
       <x:c r="W83" s="0">
         <x:v>1</x:v>
@@ -4549,7 +4549,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="I84" s="0">
-        <x:v>440</x:v>
+        <x:v>1E-06</x:v>
       </x:c>
       <x:c r="W84" s="0">
         <x:v>1</x:v>
@@ -4572,7 +4572,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="I85" s="0">
-        <x:v>10.13</x:v>
+        <x:v>1E-06</x:v>
       </x:c>
       <x:c r="W85" s="0">
         <x:v>1</x:v>
@@ -4595,7 +4595,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="I86" s="0">
-        <x:v>15.72</x:v>
+        <x:v>1E-06</x:v>
       </x:c>
       <x:c r="W86" s="0">
         <x:v>1</x:v>
@@ -4618,7 +4618,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="I87" s="0">
-        <x:v>17.08</x:v>
+        <x:v>1E-06</x:v>
       </x:c>
       <x:c r="W87" s="0">
         <x:v>1</x:v>
@@ -4641,7 +4641,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="I88" s="0">
-        <x:v>0.03</x:v>
+        <x:v>1E-06</x:v>
       </x:c>
       <x:c r="W88" s="0">
         <x:v>1</x:v>
@@ -4664,7 +4664,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="I89" s="0">
-        <x:v>0.03</x:v>
+        <x:v>1E-06</x:v>
       </x:c>
       <x:c r="W89" s="0">
         <x:v>1</x:v>
@@ -4687,7 +4687,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="I90" s="0">
-        <x:v>0.03</x:v>
+        <x:v>1E-06</x:v>
       </x:c>
       <x:c r="W90" s="0">
         <x:v>1</x:v>
@@ -4710,7 +4710,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="I91" s="0">
-        <x:v>54.72</x:v>
+        <x:v>1E-06</x:v>
       </x:c>
       <x:c r="W91" s="0">
         <x:v>1</x:v>
@@ -4733,7 +4733,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="I92" s="0">
-        <x:v>39.12</x:v>
+        <x:v>1E-06</x:v>
       </x:c>
       <x:c r="W92" s="0">
         <x:v>1</x:v>
@@ -4756,7 +4756,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="I93" s="0">
-        <x:v>34.22</x:v>
+        <x:v>1E-06</x:v>
       </x:c>
       <x:c r="W93" s="0">
         <x:v>1</x:v>
@@ -4779,7 +4779,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="I94" s="0">
-        <x:v>0</x:v>
+        <x:v>1E-06</x:v>
       </x:c>
       <x:c r="W94" s="0">
         <x:v>1</x:v>
@@ -4802,7 +4802,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="I95" s="0">
-        <x:v>1.1</x:v>
+        <x:v>1E-06</x:v>
       </x:c>
       <x:c r="W95" s="0">
         <x:v>1</x:v>
@@ -4825,7 +4825,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="I96" s="0">
-        <x:v>0</x:v>
+        <x:v>1E-06</x:v>
       </x:c>
       <x:c r="W96" s="0">
         <x:v>1</x:v>
@@ -4848,7 +4848,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="I97" s="0">
-        <x:v>2.09</x:v>
+        <x:v>1E-06</x:v>
       </x:c>
       <x:c r="W97" s="0">
         <x:v>1</x:v>
@@ -4871,7 +4871,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="I98" s="0">
-        <x:v>0</x:v>
+        <x:v>1E-06</x:v>
       </x:c>
       <x:c r="W98" s="0">
         <x:v>1</x:v>
@@ -4894,7 +4894,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="I99" s="0">
-        <x:v>33.47</x:v>
+        <x:v>1E-06</x:v>
       </x:c>
       <x:c r="W99" s="0">
         <x:v>1</x:v>
@@ -4917,7 +4917,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="I100" s="0">
-        <x:v>0</x:v>
+        <x:v>1E-06</x:v>
       </x:c>
       <x:c r="W100" s="0">
         <x:v>1</x:v>
@@ -4940,7 +4940,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="I101" s="0">
-        <x:v>0.03</x:v>
+        <x:v>1E-06</x:v>
       </x:c>
       <x:c r="W101" s="0">
         <x:v>1</x:v>
@@ -4963,7 +4963,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="I102" s="0">
-        <x:v>0.03</x:v>
+        <x:v>1E-06</x:v>
       </x:c>
       <x:c r="W102" s="0">
         <x:v>1</x:v>
@@ -4986,7 +4986,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="I103" s="0">
-        <x:v>2.63</x:v>
+        <x:v>1E-06</x:v>
       </x:c>
       <x:c r="W103" s="0">
         <x:v>1</x:v>
@@ -5009,7 +5009,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="I104" s="0">
-        <x:v>0.03</x:v>
+        <x:v>1E-06</x:v>
       </x:c>
       <x:c r="W104" s="0">
         <x:v>1</x:v>
@@ -5032,7 +5032,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="I105" s="0">
-        <x:v>0.03</x:v>
+        <x:v>1E-06</x:v>
       </x:c>
       <x:c r="W105" s="0">
         <x:v>1</x:v>
@@ -5055,7 +5055,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="I106" s="0">
-        <x:v>0.71</x:v>
+        <x:v>1E-06</x:v>
       </x:c>
       <x:c r="W106" s="0">
         <x:v>1</x:v>
@@ -5078,7 +5078,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="I107" s="0">
-        <x:v>133.28</x:v>
+        <x:v>1E-06</x:v>
       </x:c>
       <x:c r="W107" s="0">
         <x:v>1</x:v>
@@ -5124,7 +5124,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="I109" s="0">
-        <x:v>649.02</x:v>
+        <x:v>1E-06</x:v>
       </x:c>
       <x:c r="W109" s="0">
         <x:v>1</x:v>
@@ -5147,7 +5147,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="I110" s="0">
-        <x:v>0.58</x:v>
+        <x:v>1E-06</x:v>
       </x:c>
       <x:c r="W110" s="0">
         <x:v>1</x:v>
@@ -5170,7 +5170,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="I111" s="0">
-        <x:v>0.03</x:v>
+        <x:v>1E-06</x:v>
       </x:c>
       <x:c r="W111" s="0">
         <x:v>1</x:v>
@@ -5193,7 +5193,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="I112" s="0">
-        <x:v>173.42</x:v>
+        <x:v>1E-06</x:v>
       </x:c>
       <x:c r="W112" s="0">
         <x:v>1</x:v>
@@ -5216,7 +5216,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="I113" s="0">
-        <x:v>0.03</x:v>
+        <x:v>1E-06</x:v>
       </x:c>
       <x:c r="W113" s="0">
         <x:v>1</x:v>
@@ -5239,7 +5239,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="I114" s="0">
-        <x:v>0</x:v>
+        <x:v>1E-06</x:v>
       </x:c>
       <x:c r="W114" s="0">
         <x:v>1</x:v>
@@ -5262,7 +5262,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="I115" s="0">
-        <x:v>22.62</x:v>
+        <x:v>1E-06</x:v>
       </x:c>
       <x:c r="W115" s="0">
         <x:v>1</x:v>
@@ -5285,7 +5285,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="I116" s="0">
-        <x:v>144.42</x:v>
+        <x:v>1E-06</x:v>
       </x:c>
       <x:c r="W116" s="0">
         <x:v>1</x:v>
@@ -5308,7 +5308,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="I117" s="0">
-        <x:v>927.99</x:v>
+        <x:v>1E-06</x:v>
       </x:c>
       <x:c r="W117" s="0">
         <x:v>1</x:v>
@@ -5331,7 +5331,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="I118" s="0">
-        <x:v>319</x:v>
+        <x:v>1E-06</x:v>
       </x:c>
       <x:c r="W118" s="0">
         <x:v>1</x:v>
@@ -5354,7 +5354,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="I119" s="0">
-        <x:v>8.87</x:v>
+        <x:v>1E-06</x:v>
       </x:c>
       <x:c r="W119" s="0">
         <x:v>1</x:v>
@@ -5377,7 +5377,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="I120" s="0">
-        <x:v>0.03</x:v>
+        <x:v>1E-06</x:v>
       </x:c>
       <x:c r="W120" s="0">
         <x:v>1</x:v>
@@ -5400,7 +5400,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="I121" s="0">
-        <x:v>16.82</x:v>
+        <x:v>1E-06</x:v>
       </x:c>
       <x:c r="W121" s="0">
         <x:v>1</x:v>
@@ -5423,7 +5423,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="I122" s="0">
-        <x:v>0.03</x:v>
+        <x:v>1E-06</x:v>
       </x:c>
       <x:c r="W122" s="0">
         <x:v>1</x:v>
@@ -5446,7 +5446,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="I123" s="0">
-        <x:v>0.03</x:v>
+        <x:v>1E-06</x:v>
       </x:c>
       <x:c r="W123" s="0">
         <x:v>1</x:v>
@@ -5469,7 +5469,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="I124" s="0">
-        <x:v>0.03</x:v>
+        <x:v>1E-06</x:v>
       </x:c>
       <x:c r="W124" s="0">
         <x:v>1</x:v>
@@ -5492,7 +5492,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="I125" s="0">
-        <x:v>28.42</x:v>
+        <x:v>1E-06</x:v>
       </x:c>
       <x:c r="W125" s="0">
         <x:v>1</x:v>
@@ -5515,7 +5515,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="I126" s="0">
-        <x:v>11.02</x:v>
+        <x:v>1E-06</x:v>
       </x:c>
       <x:c r="W126" s="0">
         <x:v>1</x:v>
@@ -5538,7 +5538,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="I127" s="0">
-        <x:v>28.42</x:v>
+        <x:v>1E-06</x:v>
       </x:c>
       <x:c r="W127" s="0">
         <x:v>1</x:v>
@@ -5561,7 +5561,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="I128" s="0">
-        <x:v>0</x:v>
+        <x:v>1E-06</x:v>
       </x:c>
       <x:c r="W128" s="0">
         <x:v>1</x:v>
@@ -5584,7 +5584,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="I129" s="0">
-        <x:v>3.18</x:v>
+        <x:v>1E-06</x:v>
       </x:c>
       <x:c r="W129" s="0">
         <x:v>1</x:v>
@@ -5607,7 +5607,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="I130" s="0">
-        <x:v>0</x:v>
+        <x:v>1E-06</x:v>
       </x:c>
       <x:c r="W130" s="0">
         <x:v>1</x:v>
@@ -5630,7 +5630,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="I131" s="0">
-        <x:v>2.16</x:v>
+        <x:v>1E-06</x:v>
       </x:c>
       <x:c r="W131" s="0">
         <x:v>1</x:v>
@@ -5653,7 +5653,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="I132" s="0">
-        <x:v>0</x:v>
+        <x:v>1E-06</x:v>
       </x:c>
       <x:c r="W132" s="0">
         <x:v>1</x:v>
@@ -5676,7 +5676,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="I133" s="0">
-        <x:v>45.82</x:v>
+        <x:v>1E-06</x:v>
       </x:c>
       <x:c r="W133" s="0">
         <x:v>1</x:v>
@@ -5699,7 +5699,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="I134" s="0">
-        <x:v>0</x:v>
+        <x:v>1E-06</x:v>
       </x:c>
       <x:c r="W134" s="0">
         <x:v>1</x:v>
@@ -5722,7 +5722,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="I135" s="0">
-        <x:v>0.03</x:v>
+        <x:v>1E-06</x:v>
       </x:c>
       <x:c r="W135" s="0">
         <x:v>1</x:v>
@@ -5745,7 +5745,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="I136" s="0">
-        <x:v>0.03</x:v>
+        <x:v>1E-06</x:v>
       </x:c>
       <x:c r="W136" s="0">
         <x:v>1</x:v>
@@ -5768,7 +5768,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="I137" s="0">
-        <x:v>3.06</x:v>
+        <x:v>1E-06</x:v>
       </x:c>
       <x:c r="W137" s="0">
         <x:v>1</x:v>
@@ -5791,7 +5791,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="I138" s="0">
-        <x:v>0.03</x:v>
+        <x:v>1E-06</x:v>
       </x:c>
       <x:c r="W138" s="0">
         <x:v>1</x:v>
@@ -5814,7 +5814,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="I139" s="0">
-        <x:v>0.77</x:v>
+        <x:v>1E-06</x:v>
       </x:c>
       <x:c r="W139" s="0">
         <x:v>1</x:v>
@@ -5837,7 +5837,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="I140" s="0">
-        <x:v>96.01</x:v>
+        <x:v>1E-06</x:v>
       </x:c>
       <x:c r="W140" s="0">
         <x:v>1</x:v>
@@ -5883,7 +5883,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="I142" s="0">
-        <x:v>769.84</x:v>
+        <x:v>1E-06</x:v>
       </x:c>
       <x:c r="W142" s="0">
         <x:v>1</x:v>
@@ -5906,7 +5906,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="I143" s="0">
-        <x:v>0.03</x:v>
+        <x:v>1E-06</x:v>
       </x:c>
       <x:c r="W143" s="0">
         <x:v>1</x:v>
@@ -5929,7 +5929,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="I144" s="0">
-        <x:v>0.03</x:v>
+        <x:v>1E-06</x:v>
       </x:c>
       <x:c r="W144" s="0">
         <x:v>1</x:v>
@@ -5952,7 +5952,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="I145" s="0">
-        <x:v>258.2</x:v>
+        <x:v>1E-06</x:v>
       </x:c>
       <x:c r="W145" s="0">
         <x:v>1</x:v>
@@ -5975,7 +5975,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="I146" s="0">
-        <x:v>0.03</x:v>
+        <x:v>1E-06</x:v>
       </x:c>
       <x:c r="W146" s="0">
         <x:v>1</x:v>
@@ -5998,7 +5998,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="I147" s="0">
-        <x:v>0</x:v>
+        <x:v>1E-06</x:v>
       </x:c>
       <x:c r="W147" s="0">
         <x:v>1</x:v>
@@ -6021,7 +6021,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="I148" s="0">
-        <x:v>30.8</x:v>
+        <x:v>1E-06</x:v>
       </x:c>
       <x:c r="W148" s="0">
         <x:v>1</x:v>
@@ -6044,7 +6044,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="I149" s="0">
-        <x:v>123.79</x:v>
+        <x:v>1E-06</x:v>
       </x:c>
       <x:c r="W149" s="0">
         <x:v>1</x:v>
@@ -6067,7 +6067,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="I150" s="0">
-        <x:v>1069.92</x:v>
+        <x:v>1E-06</x:v>
       </x:c>
       <x:c r="W150" s="0">
         <x:v>1</x:v>
@@ -6090,7 +6090,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="I151" s="0">
-        <x:v>440</x:v>
+        <x:v>1E-06</x:v>
       </x:c>
       <x:c r="W151" s="0">
         <x:v>1</x:v>
@@ -6113,7 +6113,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="I152" s="0">
-        <x:v>10.13</x:v>
+        <x:v>1E-06</x:v>
       </x:c>
       <x:c r="W152" s="0">
         <x:v>1</x:v>
@@ -6136,7 +6136,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="I153" s="0">
-        <x:v>15.72</x:v>
+        <x:v>1E-06</x:v>
       </x:c>
       <x:c r="W153" s="0">
         <x:v>1</x:v>
@@ -6159,7 +6159,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="I154" s="0">
-        <x:v>17.08</x:v>
+        <x:v>1E-06</x:v>
       </x:c>
       <x:c r="W154" s="0">
         <x:v>1</x:v>
@@ -6182,7 +6182,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="I155" s="0">
-        <x:v>0.03</x:v>
+        <x:v>1E-06</x:v>
       </x:c>
       <x:c r="W155" s="0">
         <x:v>1</x:v>
@@ -6205,7 +6205,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="I156" s="0">
-        <x:v>0.03</x:v>
+        <x:v>1E-06</x:v>
       </x:c>
       <x:c r="W156" s="0">
         <x:v>1</x:v>
@@ -6228,7 +6228,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="I157" s="0">
-        <x:v>0.03</x:v>
+        <x:v>1E-06</x:v>
       </x:c>
       <x:c r="W157" s="0">
         <x:v>1</x:v>
@@ -6251,7 +6251,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="I158" s="0">
-        <x:v>49.69</x:v>
+        <x:v>1E-06</x:v>
       </x:c>
       <x:c r="W158" s="0">
         <x:v>1</x:v>
@@ -6274,7 +6274,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="I159" s="0">
-        <x:v>39.12</x:v>
+        <x:v>1E-06</x:v>
       </x:c>
       <x:c r="W159" s="0">
         <x:v>1</x:v>
@@ -6297,7 +6297,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="I160" s="0">
-        <x:v>34.22</x:v>
+        <x:v>1E-06</x:v>
       </x:c>
       <x:c r="W160" s="0">
         <x:v>1</x:v>
@@ -6320,7 +6320,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="I161" s="0">
-        <x:v>0</x:v>
+        <x:v>1E-06</x:v>
       </x:c>
       <x:c r="W161" s="0">
         <x:v>1</x:v>
@@ -6343,7 +6343,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="I162" s="0">
-        <x:v>1.1</x:v>
+        <x:v>1E-06</x:v>
       </x:c>
       <x:c r="W162" s="0">
         <x:v>1</x:v>
@@ -6366,7 +6366,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="I163" s="0">
-        <x:v>0</x:v>
+        <x:v>1E-06</x:v>
       </x:c>
       <x:c r="W163" s="0">
         <x:v>1</x:v>
@@ -6389,7 +6389,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="I164" s="0">
-        <x:v>2.09</x:v>
+        <x:v>1E-06</x:v>
       </x:c>
       <x:c r="W164" s="0">
         <x:v>1</x:v>
@@ -6412,7 +6412,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="I165" s="0">
-        <x:v>0</x:v>
+        <x:v>1E-06</x:v>
       </x:c>
       <x:c r="W165" s="0">
         <x:v>1</x:v>
@@ -6435,7 +6435,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="I166" s="0">
-        <x:v>33.47</x:v>
+        <x:v>1E-06</x:v>
       </x:c>
       <x:c r="W166" s="0">
         <x:v>1</x:v>
@@ -6458,7 +6458,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="I167" s="0">
-        <x:v>0</x:v>
+        <x:v>1E-06</x:v>
       </x:c>
       <x:c r="W167" s="0">
         <x:v>1</x:v>
@@ -6481,7 +6481,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="I168" s="0">
-        <x:v>0.03</x:v>
+        <x:v>1E-06</x:v>
       </x:c>
       <x:c r="W168" s="0">
         <x:v>1</x:v>
@@ -6504,7 +6504,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="I169" s="0">
-        <x:v>0.03</x:v>
+        <x:v>1E-06</x:v>
       </x:c>
       <x:c r="W169" s="0">
         <x:v>1</x:v>
@@ -6527,7 +6527,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="I170" s="0">
-        <x:v>2.63</x:v>
+        <x:v>1E-06</x:v>
       </x:c>
       <x:c r="W170" s="0">
         <x:v>1</x:v>
@@ -6550,7 +6550,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="I171" s="0">
-        <x:v>0.03</x:v>
+        <x:v>1E-06</x:v>
       </x:c>
       <x:c r="W171" s="0">
         <x:v>1</x:v>
@@ -6573,7 +6573,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="I172" s="0">
-        <x:v>0.03</x:v>
+        <x:v>1E-06</x:v>
       </x:c>
       <x:c r="W172" s="0">
         <x:v>1</x:v>
@@ -6596,7 +6596,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="I173" s="0">
-        <x:v>0.71</x:v>
+        <x:v>1E-06</x:v>
       </x:c>
       <x:c r="W173" s="0">
         <x:v>1</x:v>
@@ -6619,7 +6619,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="I174" s="0">
-        <x:v>90.21</x:v>
+        <x:v>1E-06</x:v>
       </x:c>
       <x:c r="W174" s="0">
         <x:v>1</x:v>
@@ -6665,7 +6665,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="I176" s="0">
-        <x:v>510.39</x:v>
+        <x:v>1E-06</x:v>
       </x:c>
       <x:c r="W176" s="0">
         <x:v>1</x:v>
@@ -6688,7 +6688,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="I177" s="0">
-        <x:v>0.58</x:v>
+        <x:v>1E-06</x:v>
       </x:c>
       <x:c r="W177" s="0">
         <x:v>1</x:v>
@@ -6711,7 +6711,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="I178" s="0">
-        <x:v>0.03</x:v>
+        <x:v>1E-06</x:v>
       </x:c>
       <x:c r="W178" s="0">
         <x:v>1</x:v>
@@ -6734,7 +6734,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="I179" s="0">
-        <x:v>173.42</x:v>
+        <x:v>1E-06</x:v>
       </x:c>
       <x:c r="W179" s="0">
         <x:v>1</x:v>
@@ -6757,7 +6757,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="I180" s="0">
-        <x:v>0.03</x:v>
+        <x:v>1E-06</x:v>
       </x:c>
       <x:c r="W180" s="0">
         <x:v>1</x:v>
@@ -6780,7 +6780,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="I181" s="0">
-        <x:v>0</x:v>
+        <x:v>1E-06</x:v>
       </x:c>
       <x:c r="W181" s="0">
         <x:v>1</x:v>
@@ -6803,7 +6803,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="I182" s="0">
-        <x:v>22.62</x:v>
+        <x:v>1E-06</x:v>
       </x:c>
       <x:c r="W182" s="0">
         <x:v>1</x:v>
@@ -6826,7 +6826,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="I183" s="0">
-        <x:v>144.42</x:v>
+        <x:v>1E-06</x:v>
       </x:c>
       <x:c r="W183" s="0">
         <x:v>1</x:v>
@@ -6849,7 +6849,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="I184" s="0">
-        <x:v>464</x:v>
+        <x:v>1E-06</x:v>
       </x:c>
       <x:c r="W184" s="0">
         <x:v>1</x:v>
@@ -6872,7 +6872,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="I185" s="0">
-        <x:v>255.2</x:v>
+        <x:v>1E-06</x:v>
       </x:c>
       <x:c r="W185" s="0">
         <x:v>1</x:v>
@@ -6895,7 +6895,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="I186" s="0">
-        <x:v>8.87</x:v>
+        <x:v>1E-06</x:v>
       </x:c>
       <x:c r="W186" s="0">
         <x:v>1</x:v>
@@ -6918,7 +6918,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="I187" s="0">
-        <x:v>0.03</x:v>
+        <x:v>1E-06</x:v>
       </x:c>
       <x:c r="W187" s="0">
         <x:v>1</x:v>
@@ -6941,7 +6941,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="I188" s="0">
-        <x:v>16.82</x:v>
+        <x:v>1E-06</x:v>
       </x:c>
       <x:c r="W188" s="0">
         <x:v>1</x:v>
@@ -6964,7 +6964,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="I189" s="0">
-        <x:v>0.03</x:v>
+        <x:v>1E-06</x:v>
       </x:c>
       <x:c r="W189" s="0">
         <x:v>1</x:v>
@@ -6987,7 +6987,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="I190" s="0">
-        <x:v>0.03</x:v>
+        <x:v>1E-06</x:v>
       </x:c>
       <x:c r="W190" s="0">
         <x:v>1</x:v>
@@ -7010,7 +7010,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="I191" s="0">
-        <x:v>0.03</x:v>
+        <x:v>1E-06</x:v>
       </x:c>
       <x:c r="W191" s="0">
         <x:v>1</x:v>
@@ -7033,7 +7033,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="I192" s="0">
-        <x:v>28.42</x:v>
+        <x:v>1E-06</x:v>
       </x:c>
       <x:c r="W192" s="0">
         <x:v>1</x:v>
@@ -7056,7 +7056,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="I193" s="0">
-        <x:v>11.02</x:v>
+        <x:v>1E-06</x:v>
       </x:c>
       <x:c r="W193" s="0">
         <x:v>1</x:v>
@@ -7079,7 +7079,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="I194" s="0">
-        <x:v>28.42</x:v>
+        <x:v>1E-06</x:v>
       </x:c>
       <x:c r="W194" s="0">
         <x:v>1</x:v>
@@ -7102,7 +7102,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="I195" s="0">
-        <x:v>0</x:v>
+        <x:v>1E-06</x:v>
       </x:c>
       <x:c r="W195" s="0">
         <x:v>1</x:v>
@@ -7125,7 +7125,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="I196" s="0">
-        <x:v>3.18</x:v>
+        <x:v>1E-06</x:v>
       </x:c>
       <x:c r="W196" s="0">
         <x:v>1</x:v>
@@ -7148,7 +7148,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="I197" s="0">
-        <x:v>0</x:v>
+        <x:v>1E-06</x:v>
       </x:c>
       <x:c r="W197" s="0">
         <x:v>1</x:v>
@@ -7171,7 +7171,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="I198" s="0">
-        <x:v>2.16</x:v>
+        <x:v>1E-06</x:v>
       </x:c>
       <x:c r="W198" s="0">
         <x:v>1</x:v>
@@ -7194,7 +7194,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="I199" s="0">
-        <x:v>0</x:v>
+        <x:v>1E-06</x:v>
       </x:c>
       <x:c r="W199" s="0">
         <x:v>1</x:v>
@@ -7217,7 +7217,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="I200" s="0">
-        <x:v>45.82</x:v>
+        <x:v>1E-06</x:v>
       </x:c>
       <x:c r="W200" s="0">
         <x:v>1</x:v>
@@ -7240,7 +7240,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="I201" s="0">
-        <x:v>0</x:v>
+        <x:v>1E-06</x:v>
       </x:c>
       <x:c r="W201" s="0">
         <x:v>1</x:v>
@@ -7263,7 +7263,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="I202" s="0">
-        <x:v>0.03</x:v>
+        <x:v>1E-06</x:v>
       </x:c>
       <x:c r="W202" s="0">
         <x:v>1</x:v>
@@ -7286,7 +7286,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="I203" s="0">
-        <x:v>0.03</x:v>
+        <x:v>1E-06</x:v>
       </x:c>
       <x:c r="W203" s="0">
         <x:v>1</x:v>
@@ -7309,7 +7309,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="I204" s="0">
-        <x:v>3.06</x:v>
+        <x:v>1E-06</x:v>
       </x:c>
       <x:c r="W204" s="0">
         <x:v>1</x:v>
@@ -7332,7 +7332,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="I205" s="0">
-        <x:v>0.03</x:v>
+        <x:v>1E-06</x:v>
       </x:c>
       <x:c r="W205" s="0">
         <x:v>1</x:v>
@@ -7355,7 +7355,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="I206" s="0">
-        <x:v>0.77</x:v>
+        <x:v>1E-06</x:v>
       </x:c>
       <x:c r="W206" s="0">
         <x:v>1</x:v>
@@ -7378,7 +7378,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="I207" s="0">
-        <x:v>96.01</x:v>
+        <x:v>1E-06</x:v>
       </x:c>
       <x:c r="W207" s="0">
         <x:v>1</x:v>
@@ -7424,7 +7424,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="I209" s="0">
-        <x:v>526.01</x:v>
+        <x:v>1E-06</x:v>
       </x:c>
       <x:c r="W209" s="0">
         <x:v>1</x:v>
@@ -7447,7 +7447,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="I210" s="0">
-        <x:v>0.6</x:v>
+        <x:v>1E-06</x:v>
       </x:c>
       <x:c r="W210" s="0">
         <x:v>1</x:v>
@@ -7470,7 +7470,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="I211" s="0">
-        <x:v>0.03</x:v>
+        <x:v>1E-06</x:v>
       </x:c>
       <x:c r="W211" s="0">
         <x:v>1</x:v>
@@ -7493,7 +7493,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="I212" s="0">
-        <x:v>178.73</x:v>
+        <x:v>1E-06</x:v>
       </x:c>
       <x:c r="W212" s="0">
         <x:v>1</x:v>
@@ -7516,7 +7516,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="I213" s="0">
-        <x:v>0.03</x:v>
+        <x:v>1E-06</x:v>
       </x:c>
       <x:c r="W213" s="0">
         <x:v>1</x:v>
@@ -7539,7 +7539,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="I214" s="0">
-        <x:v>0</x:v>
+        <x:v>1E-06</x:v>
       </x:c>
       <x:c r="W214" s="0">
         <x:v>1</x:v>
@@ -7562,7 +7562,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="I215" s="0">
-        <x:v>23.31</x:v>
+        <x:v>1E-06</x:v>
       </x:c>
       <x:c r="W215" s="0">
         <x:v>1</x:v>
@@ -7585,7 +7585,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="I216" s="0">
-        <x:v>148.84</x:v>
+        <x:v>1E-06</x:v>
       </x:c>
       <x:c r="W216" s="0">
         <x:v>1</x:v>
@@ -7608,7 +7608,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="I217" s="0">
-        <x:v>478.2</x:v>
+        <x:v>1E-06</x:v>
       </x:c>
       <x:c r="W217" s="0">
         <x:v>1</x:v>
@@ -7631,7 +7631,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="I218" s="0">
-        <x:v>263.01</x:v>
+        <x:v>1E-06</x:v>
       </x:c>
       <x:c r="W218" s="0">
         <x:v>1</x:v>
@@ -7654,7 +7654,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="I219" s="0">
-        <x:v>9.14</x:v>
+        <x:v>1E-06</x:v>
       </x:c>
       <x:c r="W219" s="0">
         <x:v>1</x:v>
@@ -7677,7 +7677,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="I220" s="0">
-        <x:v>0.03</x:v>
+        <x:v>1E-06</x:v>
       </x:c>
       <x:c r="W220" s="0">
         <x:v>1</x:v>
@@ -7700,7 +7700,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="I221" s="0">
-        <x:v>17.33</x:v>
+        <x:v>1E-06</x:v>
       </x:c>
       <x:c r="W221" s="0">
         <x:v>1</x:v>
@@ -7723,7 +7723,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="I222" s="0">
-        <x:v>0.03</x:v>
+        <x:v>1E-06</x:v>
       </x:c>
       <x:c r="W222" s="0">
         <x:v>1</x:v>
@@ -7746,7 +7746,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="I223" s="0">
-        <x:v>0.03</x:v>
+        <x:v>1E-06</x:v>
       </x:c>
       <x:c r="W223" s="0">
         <x:v>1</x:v>
@@ -7769,7 +7769,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="I224" s="0">
-        <x:v>0.03</x:v>
+        <x:v>1E-06</x:v>
       </x:c>
       <x:c r="W224" s="0">
         <x:v>1</x:v>
@@ -7792,7 +7792,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="I225" s="0">
-        <x:v>29.29</x:v>
+        <x:v>1E-06</x:v>
       </x:c>
       <x:c r="W225" s="0">
         <x:v>1</x:v>
@@ -7815,7 +7815,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="I226" s="0">
-        <x:v>11.36</x:v>
+        <x:v>1E-06</x:v>
       </x:c>
       <x:c r="W226" s="0">
         <x:v>1</x:v>
@@ -7838,7 +7838,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="I227" s="0">
-        <x:v>29.29</x:v>
+        <x:v>1E-06</x:v>
       </x:c>
       <x:c r="W227" s="0">
         <x:v>1</x:v>
@@ -7861,7 +7861,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="I228" s="0">
-        <x:v>0</x:v>
+        <x:v>1E-06</x:v>
       </x:c>
       <x:c r="W228" s="0">
         <x:v>1</x:v>
@@ -7884,7 +7884,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="I229" s="0">
-        <x:v>3.28</x:v>
+        <x:v>1E-06</x:v>
       </x:c>
       <x:c r="W229" s="0">
         <x:v>1</x:v>
@@ -7907,7 +7907,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="I230" s="0">
-        <x:v>0</x:v>
+        <x:v>1E-06</x:v>
       </x:c>
       <x:c r="W230" s="0">
         <x:v>1</x:v>
@@ -7930,7 +7930,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="I231" s="0">
-        <x:v>2.23</x:v>
+        <x:v>1E-06</x:v>
       </x:c>
       <x:c r="W231" s="0">
         <x:v>1</x:v>
@@ -7953,7 +7953,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="I232" s="0">
-        <x:v>0</x:v>
+        <x:v>1E-06</x:v>
       </x:c>
       <x:c r="W232" s="0">
         <x:v>1</x:v>
@@ -7976,7 +7976,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="I233" s="0">
-        <x:v>47.22</x:v>
+        <x:v>1E-06</x:v>
       </x:c>
       <x:c r="W233" s="0">
         <x:v>1</x:v>
@@ -7999,7 +7999,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="I234" s="0">
-        <x:v>0</x:v>
+        <x:v>1E-06</x:v>
       </x:c>
       <x:c r="W234" s="0">
         <x:v>1</x:v>
@@ -8022,7 +8022,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="I235" s="0">
-        <x:v>0.03</x:v>
+        <x:v>1E-06</x:v>
       </x:c>
       <x:c r="W235" s="0">
         <x:v>1</x:v>
@@ -8045,7 +8045,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="I236" s="0">
-        <x:v>0.03</x:v>
+        <x:v>1E-06</x:v>
       </x:c>
       <x:c r="W236" s="0">
         <x:v>1</x:v>
@@ -8068,7 +8068,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="I237" s="0">
-        <x:v>3.15</x:v>
+        <x:v>1E-06</x:v>
       </x:c>
       <x:c r="W237" s="0">
         <x:v>1</x:v>
@@ -8091,7 +8091,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="I238" s="0">
-        <x:v>0.03</x:v>
+        <x:v>1E-06</x:v>
       </x:c>
       <x:c r="W238" s="0">
         <x:v>1</x:v>
@@ -8114,7 +8114,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="I239" s="0">
-        <x:v>0.8</x:v>
+        <x:v>1E-06</x:v>
       </x:c>
       <x:c r="W239" s="0">
         <x:v>1</x:v>
@@ -8137,7 +8137,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="I240" s="0">
-        <x:v>98.94</x:v>
+        <x:v>1E-06</x:v>
       </x:c>
       <x:c r="W240" s="0">
         <x:v>1</x:v>
@@ -8183,7 +8183,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="I242" s="0">
-        <x:v>827.92</x:v>
+        <x:v>1E-06</x:v>
       </x:c>
       <x:c r="W242" s="0">
         <x:v>1</x:v>
@@ -8206,7 +8206,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="I243" s="0">
-        <x:v>0.48</x:v>
+        <x:v>1E-06</x:v>
       </x:c>
       <x:c r="W243" s="0">
         <x:v>1</x:v>
@@ -8229,7 +8229,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="I244" s="0">
-        <x:v>0.02</x:v>
+        <x:v>1E-06</x:v>
       </x:c>
       <x:c r="W244" s="0">
         <x:v>1</x:v>
@@ -8252,7 +8252,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="I245" s="0">
-        <x:v>277.36</x:v>
+        <x:v>1E-06</x:v>
       </x:c>
       <x:c r="W245" s="0">
         <x:v>1</x:v>
@@ -8275,7 +8275,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="I246" s="0">
-        <x:v>0.02</x:v>
+        <x:v>1E-06</x:v>
       </x:c>
       <x:c r="W246" s="0">
         <x:v>1</x:v>
@@ -8298,7 +8298,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="I247" s="0">
-        <x:v>0</x:v>
+        <x:v>1E-06</x:v>
       </x:c>
       <x:c r="W247" s="0">
         <x:v>1</x:v>
@@ -8321,7 +8321,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="I248" s="0">
-        <x:v>26.1</x:v>
+        <x:v>1E-06</x:v>
       </x:c>
       <x:c r="W248" s="0">
         <x:v>1</x:v>
@@ -8344,7 +8344,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="I249" s="0">
-        <x:v>132.97</x:v>
+        <x:v>1E-06</x:v>
       </x:c>
       <x:c r="W249" s="0">
         <x:v>1</x:v>
@@ -8367,7 +8367,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="I250" s="0">
-        <x:v>765.68</x:v>
+        <x:v>1E-06</x:v>
       </x:c>
       <x:c r="W250" s="0">
         <x:v>1</x:v>
@@ -8390,7 +8390,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="I251" s="0">
-        <x:v>263.2</x:v>
+        <x:v>1E-06</x:v>
       </x:c>
       <x:c r="W251" s="0">
         <x:v>1</x:v>
@@ -8413,7 +8413,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="I252" s="0">
-        <x:v>8.94</x:v>
+        <x:v>1E-06</x:v>
       </x:c>
       <x:c r="W252" s="0">
         <x:v>1</x:v>
@@ -8436,7 +8436,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="I253" s="0">
-        <x:v>13.58</x:v>
+        <x:v>1E-06</x:v>
       </x:c>
       <x:c r="W253" s="0">
         <x:v>1</x:v>
@@ -8459,7 +8459,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="I254" s="0">
-        <x:v>14.74</x:v>
+        <x:v>1E-06</x:v>
       </x:c>
       <x:c r="W254" s="0">
         <x:v>1</x:v>
@@ -8482,7 +8482,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="I255" s="0">
-        <x:v>0.02</x:v>
+        <x:v>1E-06</x:v>
       </x:c>
       <x:c r="W255" s="0">
         <x:v>1</x:v>
@@ -8505,7 +8505,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="I256" s="0">
-        <x:v>0.02</x:v>
+        <x:v>1E-06</x:v>
       </x:c>
       <x:c r="W256" s="0">
         <x:v>1</x:v>
@@ -8528,7 +8528,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="I257" s="0">
-        <x:v>0.02</x:v>
+        <x:v>1E-06</x:v>
       </x:c>
       <x:c r="W257" s="0">
         <x:v>1</x:v>
@@ -8551,7 +8551,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="I258" s="0">
-        <x:v>58.35</x:v>
+        <x:v>1E-06</x:v>
       </x:c>
       <x:c r="W258" s="0">
         <x:v>1</x:v>
@@ -8574,7 +8574,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="I259" s="0">
-        <x:v>31.44</x:v>
+        <x:v>1E-06</x:v>
       </x:c>
       <x:c r="W259" s="0">
         <x:v>1</x:v>
@@ -8597,7 +8597,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="I260" s="0">
-        <x:v>29.54</x:v>
+        <x:v>1E-06</x:v>
       </x:c>
       <x:c r="W260" s="0">
         <x:v>1</x:v>
@@ -8620,7 +8620,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="I261" s="0">
-        <x:v>0</x:v>
+        <x:v>1E-06</x:v>
       </x:c>
       <x:c r="W261" s="0">
         <x:v>1</x:v>
@@ -8643,7 +8643,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="I262" s="0">
-        <x:v>3.75</x:v>
+        <x:v>1E-06</x:v>
       </x:c>
       <x:c r="W262" s="0">
         <x:v>1</x:v>
@@ -8666,7 +8666,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="I263" s="0">
-        <x:v>0</x:v>
+        <x:v>1E-06</x:v>
       </x:c>
       <x:c r="W263" s="0">
         <x:v>1</x:v>
@@ -8689,7 +8689,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="I264" s="0">
-        <x:v>1.91</x:v>
+        <x:v>1E-06</x:v>
       </x:c>
       <x:c r="W264" s="0">
         <x:v>1</x:v>
@@ -8712,7 +8712,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="I265" s="0">
-        <x:v>0</x:v>
+        <x:v>1E-06</x:v>
       </x:c>
       <x:c r="W265" s="0">
         <x:v>1</x:v>
@@ -8735,7 +8735,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="I266" s="0">
-        <x:v>32.74</x:v>
+        <x:v>1E-06</x:v>
       </x:c>
       <x:c r="W266" s="0">
         <x:v>1</x:v>
@@ -8758,7 +8758,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="I267" s="0">
-        <x:v>0</x:v>
+        <x:v>1E-06</x:v>
       </x:c>
       <x:c r="W267" s="0">
         <x:v>1</x:v>
@@ -8781,7 +8781,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="I268" s="0">
-        <x:v>0.02</x:v>
+        <x:v>1E-06</x:v>
       </x:c>
       <x:c r="W268" s="0">
         <x:v>1</x:v>
@@ -8804,7 +8804,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="I269" s="0">
-        <x:v>0.02</x:v>
+        <x:v>1E-06</x:v>
       </x:c>
       <x:c r="W269" s="0">
         <x:v>1</x:v>
@@ -8827,7 +8827,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="I270" s="0">
-        <x:v>2.27</x:v>
+        <x:v>1E-06</x:v>
       </x:c>
       <x:c r="W270" s="0">
         <x:v>1</x:v>
@@ -8850,7 +8850,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="I271" s="0">
-        <x:v>0.02</x:v>
+        <x:v>1E-06</x:v>
       </x:c>
       <x:c r="W271" s="0">
         <x:v>1</x:v>
@@ -8873,7 +8873,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="I272" s="0">
-        <x:v>0.02</x:v>
+        <x:v>1E-06</x:v>
       </x:c>
       <x:c r="W272" s="0">
         <x:v>1</x:v>
@@ -8896,7 +8896,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="I273" s="0">
-        <x:v>0.64</x:v>
+        <x:v>1E-06</x:v>
       </x:c>
       <x:c r="W273" s="0">
         <x:v>1</x:v>
@@ -8919,7 +8919,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="I274" s="0">
-        <x:v>79.21</x:v>
+        <x:v>1E-06</x:v>
       </x:c>
       <x:c r="W274" s="0">
         <x:v>1</x:v>
@@ -8965,7 +8965,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="I276" s="0">
-        <x:v>648.01</x:v>
+        <x:v>1E-06</x:v>
       </x:c>
       <x:c r="W276" s="0">
         <x:v>1</x:v>
@@ -8988,7 +8988,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="I277" s="0">
-        <x:v>0.58</x:v>
+        <x:v>1E-06</x:v>
       </x:c>
       <x:c r="W277" s="0">
         <x:v>1</x:v>
@@ -9011,7 +9011,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="I278" s="0">
-        <x:v>0.03</x:v>
+        <x:v>1E-06</x:v>
       </x:c>
       <x:c r="W278" s="0">
         <x:v>1</x:v>
@@ -9034,7 +9034,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="I279" s="0">
-        <x:v>173.15</x:v>
+        <x:v>1E-06</x:v>
       </x:c>
       <x:c r="W279" s="0">
         <x:v>1</x:v>
@@ -9057,7 +9057,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="I280" s="0">
-        <x:v>0.03</x:v>
+        <x:v>1E-06</x:v>
       </x:c>
       <x:c r="W280" s="0">
         <x:v>1</x:v>
@@ -9080,7 +9080,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="I281" s="0">
-        <x:v>0</x:v>
+        <x:v>1E-06</x:v>
       </x:c>
       <x:c r="W281" s="0">
         <x:v>1</x:v>
@@ -9103,7 +9103,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="I282" s="0">
-        <x:v>22.58</x:v>
+        <x:v>1E-06</x:v>
       </x:c>
       <x:c r="W282" s="0">
         <x:v>1</x:v>
@@ -9126,7 +9126,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="I283" s="0">
-        <x:v>144.19</x:v>
+        <x:v>1E-06</x:v>
       </x:c>
       <x:c r="W283" s="0">
         <x:v>1</x:v>
@@ -9149,7 +9149,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="I284" s="0">
-        <x:v>926.55</x:v>
+        <x:v>1E-06</x:v>
       </x:c>
       <x:c r="W284" s="0">
         <x:v>1</x:v>
@@ -9172,7 +9172,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="I285" s="0">
-        <x:v>318.5</x:v>
+        <x:v>1E-06</x:v>
       </x:c>
       <x:c r="W285" s="0">
         <x:v>1</x:v>
@@ -9195,7 +9195,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="I286" s="0">
-        <x:v>8.85</x:v>
+        <x:v>1E-06</x:v>
       </x:c>
       <x:c r="W286" s="0">
         <x:v>1</x:v>
@@ -9218,7 +9218,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="I287" s="0">
-        <x:v>0.03</x:v>
+        <x:v>1E-06</x:v>
       </x:c>
       <x:c r="W287" s="0">
         <x:v>1</x:v>
@@ -9241,7 +9241,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="I288" s="0">
-        <x:v>16.79</x:v>
+        <x:v>1E-06</x:v>
       </x:c>
       <x:c r="W288" s="0">
         <x:v>1</x:v>
@@ -9264,7 +9264,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="I289" s="0">
-        <x:v>0.03</x:v>
+        <x:v>1E-06</x:v>
       </x:c>
       <x:c r="W289" s="0">
         <x:v>1</x:v>
@@ -9287,7 +9287,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="I290" s="0">
-        <x:v>0.03</x:v>
+        <x:v>1E-06</x:v>
       </x:c>
       <x:c r="W290" s="0">
         <x:v>1</x:v>
@@ -9310,7 +9310,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="I291" s="0">
-        <x:v>0.03</x:v>
+        <x:v>1E-06</x:v>
       </x:c>
       <x:c r="W291" s="0">
         <x:v>1</x:v>
@@ -9333,7 +9333,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="I292" s="0">
-        <x:v>28.38</x:v>
+        <x:v>1E-06</x:v>
       </x:c>
       <x:c r="W292" s="0">
         <x:v>1</x:v>
@@ -9356,7 +9356,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="I293" s="0">
-        <x:v>11</x:v>
+        <x:v>1E-06</x:v>
       </x:c>
       <x:c r="W293" s="0">
         <x:v>1</x:v>
@@ -9379,7 +9379,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="I294" s="0">
-        <x:v>28.38</x:v>
+        <x:v>1E-06</x:v>
       </x:c>
       <x:c r="W294" s="0">
         <x:v>1</x:v>
@@ -9402,7 +9402,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="I295" s="0">
-        <x:v>0</x:v>
+        <x:v>1E-06</x:v>
       </x:c>
       <x:c r="W295" s="0">
         <x:v>1</x:v>
@@ -9425,7 +9425,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="I296" s="0">
-        <x:v>3.18</x:v>
+        <x:v>1E-06</x:v>
       </x:c>
       <x:c r="W296" s="0">
         <x:v>1</x:v>
@@ -9448,7 +9448,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="I297" s="0">
-        <x:v>0</x:v>
+        <x:v>1E-06</x:v>
       </x:c>
       <x:c r="W297" s="0">
         <x:v>1</x:v>
@@ -9471,7 +9471,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="I298" s="0">
-        <x:v>2.16</x:v>
+        <x:v>1E-06</x:v>
       </x:c>
       <x:c r="W298" s="0">
         <x:v>1</x:v>
@@ -9494,7 +9494,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="I299" s="0">
-        <x:v>0</x:v>
+        <x:v>1E-06</x:v>
       </x:c>
       <x:c r="W299" s="0">
         <x:v>1</x:v>
@@ -9517,7 +9517,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="I300" s="0">
-        <x:v>45.75</x:v>
+        <x:v>1E-06</x:v>
       </x:c>
       <x:c r="W300" s="0">
         <x:v>1</x:v>
@@ -9540,7 +9540,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="I301" s="0">
-        <x:v>0</x:v>
+        <x:v>1E-06</x:v>
       </x:c>
       <x:c r="W301" s="0">
         <x:v>1</x:v>
@@ -9563,7 +9563,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="I302" s="0">
-        <x:v>0.03</x:v>
+        <x:v>1E-06</x:v>
       </x:c>
       <x:c r="W302" s="0">
         <x:v>1</x:v>
@@ -9586,7 +9586,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="I303" s="0">
-        <x:v>0.03</x:v>
+        <x:v>1E-06</x:v>
       </x:c>
       <x:c r="W303" s="0">
         <x:v>1</x:v>
@@ -9609,7 +9609,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="I304" s="0">
-        <x:v>3.05</x:v>
+        <x:v>1E-06</x:v>
       </x:c>
       <x:c r="W304" s="0">
         <x:v>1</x:v>
@@ -9632,7 +9632,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="I305" s="0">
-        <x:v>0.03</x:v>
+        <x:v>1E-06</x:v>
       </x:c>
       <x:c r="W305" s="0">
         <x:v>1</x:v>
@@ -9655,7 +9655,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="I306" s="0">
-        <x:v>0.77</x:v>
+        <x:v>1E-06</x:v>
       </x:c>
       <x:c r="W306" s="0">
         <x:v>1</x:v>
@@ -9678,7 +9678,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="I307" s="0">
-        <x:v>95.86</x:v>
+        <x:v>1E-06</x:v>
       </x:c>
       <x:c r="W307" s="0">
         <x:v>1</x:v>
@@ -9724,7 +9724,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="I309" s="0">
-        <x:v>637.48</x:v>
+        <x:v>1E-06</x:v>
       </x:c>
       <x:c r="W309" s="0">
         <x:v>1</x:v>
@@ -9747,7 +9747,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="I310" s="0">
-        <x:v>0.47</x:v>
+        <x:v>1E-06</x:v>
       </x:c>
       <x:c r="W310" s="0">
         <x:v>1</x:v>
@@ -9770,7 +9770,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="I311" s="0">
-        <x:v>0.02</x:v>
+        <x:v>1E-06</x:v>
       </x:c>
       <x:c r="W311" s="0">
         <x:v>1</x:v>
@@ -9793,7 +9793,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="I312" s="0">
-        <x:v>271.91</x:v>
+        <x:v>1E-06</x:v>
       </x:c>
       <x:c r="W312" s="0">
         <x:v>1</x:v>
@@ -9816,7 +9816,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="I313" s="0">
-        <x:v>0.02</x:v>
+        <x:v>1E-06</x:v>
       </x:c>
       <x:c r="W313" s="0">
         <x:v>1</x:v>
@@ -9839,7 +9839,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="I314" s="0">
-        <x:v>0</x:v>
+        <x:v>1E-06</x:v>
       </x:c>
       <x:c r="W314" s="0">
         <x:v>1</x:v>
@@ -9862,7 +9862,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="I315" s="0">
-        <x:v>25.59</x:v>
+        <x:v>1E-06</x:v>
       </x:c>
       <x:c r="W315" s="0">
         <x:v>1</x:v>
@@ -9885,7 +9885,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="I316" s="0">
-        <x:v>130.36</x:v>
+        <x:v>1E-06</x:v>
       </x:c>
       <x:c r="W316" s="0">
         <x:v>1</x:v>
@@ -9908,7 +9908,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="I317" s="0">
-        <x:v>375.32</x:v>
+        <x:v>1E-06</x:v>
       </x:c>
       <x:c r="W317" s="0">
         <x:v>1</x:v>
@@ -9931,7 +9931,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="I318" s="0">
-        <x:v>258.03</x:v>
+        <x:v>1E-06</x:v>
       </x:c>
       <x:c r="W318" s="0">
         <x:v>1</x:v>
@@ -9954,7 +9954,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="I319" s="0">
-        <x:v>8.77</x:v>
+        <x:v>1E-06</x:v>
       </x:c>
       <x:c r="W319" s="0">
         <x:v>1</x:v>
@@ -9977,7 +9977,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="I320" s="0">
-        <x:v>13.31</x:v>
+        <x:v>1E-06</x:v>
       </x:c>
       <x:c r="W320" s="0">
         <x:v>1</x:v>
@@ -10000,7 +10000,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="I321" s="0">
-        <x:v>14.45</x:v>
+        <x:v>1E-06</x:v>
       </x:c>
       <x:c r="W321" s="0">
         <x:v>1</x:v>
@@ -10023,7 +10023,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="I322" s="0">
-        <x:v>0.02</x:v>
+        <x:v>1E-06</x:v>
       </x:c>
       <x:c r="W322" s="0">
         <x:v>1</x:v>
@@ -10046,7 +10046,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="I323" s="0">
-        <x:v>0.02</x:v>
+        <x:v>1E-06</x:v>
       </x:c>
       <x:c r="W323" s="0">
         <x:v>1</x:v>
@@ -10069,7 +10069,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="I324" s="0">
-        <x:v>0.02</x:v>
+        <x:v>1E-06</x:v>
       </x:c>
       <x:c r="W324" s="0">
         <x:v>1</x:v>
@@ -10092,7 +10092,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="I325" s="0">
-        <x:v>57.2</x:v>
+        <x:v>1E-06</x:v>
       </x:c>
       <x:c r="W325" s="0">
         <x:v>1</x:v>
@@ -10115,7 +10115,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="I326" s="0">
-        <x:v>30.82</x:v>
+        <x:v>1E-06</x:v>
       </x:c>
       <x:c r="W326" s="0">
         <x:v>1</x:v>
@@ -10138,7 +10138,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="I327" s="0">
-        <x:v>28.96</x:v>
+        <x:v>1E-06</x:v>
       </x:c>
       <x:c r="W327" s="0">
         <x:v>1</x:v>
@@ -10161,7 +10161,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="I328" s="0">
-        <x:v>0</x:v>
+        <x:v>1E-06</x:v>
       </x:c>
       <x:c r="W328" s="0">
         <x:v>1</x:v>
@@ -10184,7 +10184,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="I329" s="0">
-        <x:v>3.68</x:v>
+        <x:v>1E-06</x:v>
       </x:c>
       <x:c r="W329" s="0">
         <x:v>1</x:v>
@@ -10207,7 +10207,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="I330" s="0">
-        <x:v>0</x:v>
+        <x:v>1E-06</x:v>
       </x:c>
       <x:c r="W330" s="0">
         <x:v>1</x:v>
@@ -10230,7 +10230,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="I331" s="0">
-        <x:v>1.88</x:v>
+        <x:v>1E-06</x:v>
       </x:c>
       <x:c r="W331" s="0">
         <x:v>1</x:v>
@@ -10253,7 +10253,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="I332" s="0">
-        <x:v>0</x:v>
+        <x:v>1E-06</x:v>
       </x:c>
       <x:c r="W332" s="0">
         <x:v>1</x:v>
@@ -10276,7 +10276,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="I333" s="0">
-        <x:v>32.09</x:v>
+        <x:v>1E-06</x:v>
       </x:c>
       <x:c r="W333" s="0">
         <x:v>1</x:v>
@@ -10299,7 +10299,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="I334" s="0">
-        <x:v>0</x:v>
+        <x:v>1E-06</x:v>
       </x:c>
       <x:c r="W334" s="0">
         <x:v>1</x:v>
@@ -10322,7 +10322,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="I335" s="0">
-        <x:v>0.02</x:v>
+        <x:v>1E-06</x:v>
       </x:c>
       <x:c r="W335" s="0">
         <x:v>1</x:v>
@@ -10345,7 +10345,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="I336" s="0">
-        <x:v>0.02</x:v>
+        <x:v>1E-06</x:v>
       </x:c>
       <x:c r="W336" s="0">
         <x:v>1</x:v>
@@ -10368,7 +10368,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="I337" s="0">
-        <x:v>2.22</x:v>
+        <x:v>1E-06</x:v>
       </x:c>
       <x:c r="W337" s="0">
         <x:v>1</x:v>
@@ -10391,7 +10391,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="I338" s="0">
-        <x:v>0.02</x:v>
+        <x:v>1E-06</x:v>
       </x:c>
       <x:c r="W338" s="0">
         <x:v>1</x:v>
@@ -10414,7 +10414,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="I339" s="0">
-        <x:v>0.02</x:v>
+        <x:v>1E-06</x:v>
       </x:c>
       <x:c r="W339" s="0">
         <x:v>1</x:v>
@@ -10437,7 +10437,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="I340" s="0">
-        <x:v>0.62</x:v>
+        <x:v>1E-06</x:v>
       </x:c>
       <x:c r="W340" s="0">
         <x:v>1</x:v>
@@ -10460,7 +10460,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="I341" s="0">
-        <x:v>77.66</x:v>
+        <x:v>1E-06</x:v>
       </x:c>
       <x:c r="W341" s="0">
         <x:v>1</x:v>
@@ -10506,7 +10506,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="I343" s="0">
-        <x:v>924.1</x:v>
+        <x:v>1E-06</x:v>
       </x:c>
       <x:c r="W343" s="0">
         <x:v>1</x:v>
@@ -10529,7 +10529,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="I344" s="0">
-        <x:v>0.47</x:v>
+        <x:v>1E-06</x:v>
       </x:c>
       <x:c r="W344" s="0">
         <x:v>1</x:v>
@@ -10552,7 +10552,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="I345" s="0">
-        <x:v>0.02</x:v>
+        <x:v>1E-06</x:v>
       </x:c>
       <x:c r="W345" s="0">
         <x:v>1</x:v>
@@ -10575,7 +10575,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="I346" s="0">
-        <x:v>303.8</x:v>
+        <x:v>1E-06</x:v>
       </x:c>
       <x:c r="W346" s="0">
         <x:v>1</x:v>
@@ -10598,7 +10598,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="I347" s="0">
-        <x:v>0.02</x:v>
+        <x:v>1E-06</x:v>
       </x:c>
       <x:c r="W347" s="0">
         <x:v>1</x:v>
@@ -10621,7 +10621,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="I348" s="0">
-        <x:v>0</x:v>
+        <x:v>1E-06</x:v>
       </x:c>
       <x:c r="W348" s="0">
         <x:v>1</x:v>
@@ -10644,7 +10644,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="I349" s="0">
-        <x:v>25.84</x:v>
+        <x:v>1E-06</x:v>
       </x:c>
       <x:c r="W349" s="0">
         <x:v>1</x:v>
@@ -10667,7 +10667,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="I350" s="0">
-        <x:v>134.36</x:v>
+        <x:v>1E-06</x:v>
       </x:c>
       <x:c r="W350" s="0">
         <x:v>1</x:v>
@@ -10690,7 +10690,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="I351" s="0">
-        <x:v>757.97</x:v>
+        <x:v>1E-06</x:v>
       </x:c>
       <x:c r="W351" s="0">
         <x:v>1</x:v>
@@ -10713,7 +10713,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="I352" s="0">
-        <x:v>260.55</x:v>
+        <x:v>1E-06</x:v>
       </x:c>
       <x:c r="W352" s="0">
         <x:v>1</x:v>
@@ -10736,7 +10736,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="I353" s="0">
-        <x:v>0.02</x:v>
+        <x:v>1E-06</x:v>
       </x:c>
       <x:c r="W353" s="0">
         <x:v>1</x:v>
@@ -10759,7 +10759,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="I354" s="0">
-        <x:v>13.51</x:v>
+        <x:v>1E-06</x:v>
       </x:c>
       <x:c r="W354" s="0">
         <x:v>1</x:v>
@@ -10782,7 +10782,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="I355" s="0">
-        <x:v>16.36</x:v>
+        <x:v>1E-06</x:v>
       </x:c>
       <x:c r="W355" s="0">
         <x:v>1</x:v>
@@ -10805,7 +10805,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="I356" s="0">
-        <x:v>0.05</x:v>
+        <x:v>1E-06</x:v>
       </x:c>
       <x:c r="W356" s="0">
         <x:v>1</x:v>
@@ -10828,7 +10828,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="I357" s="0">
-        <x:v>1.47</x:v>
+        <x:v>1E-06</x:v>
       </x:c>
       <x:c r="W357" s="0">
         <x:v>1</x:v>
@@ -10851,7 +10851,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="I358" s="0">
-        <x:v>0.02</x:v>
+        <x:v>1E-06</x:v>
       </x:c>
       <x:c r="W358" s="0">
         <x:v>1</x:v>
@@ -10874,7 +10874,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="I359" s="0">
-        <x:v>53.01</x:v>
+        <x:v>1E-06</x:v>
       </x:c>
       <x:c r="W359" s="0">
         <x:v>1</x:v>
@@ -10897,7 +10897,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="I360" s="0">
-        <x:v>13.97</x:v>
+        <x:v>1E-06</x:v>
       </x:c>
       <x:c r="W360" s="0">
         <x:v>1</x:v>
@@ -10920,7 +10920,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="I361" s="0">
-        <x:v>33.56</x:v>
+        <x:v>1E-06</x:v>
       </x:c>
       <x:c r="W361" s="0">
         <x:v>1</x:v>
@@ -10943,7 +10943,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="I362" s="0">
-        <x:v>0</x:v>
+        <x:v>1E-06</x:v>
       </x:c>
       <x:c r="W362" s="0">
         <x:v>1</x:v>
@@ -10966,7 +10966,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="I363" s="0">
-        <x:v>3.76</x:v>
+        <x:v>1E-06</x:v>
       </x:c>
       <x:c r="W363" s="0">
         <x:v>1</x:v>
@@ -10989,7 +10989,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="I364" s="0">
-        <x:v>0</x:v>
+        <x:v>1E-06</x:v>
       </x:c>
       <x:c r="W364" s="0">
         <x:v>1</x:v>
@@ -11012,7 +11012,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="I365" s="0">
-        <x:v>1.77</x:v>
+        <x:v>1E-06</x:v>
       </x:c>
       <x:c r="W365" s="0">
         <x:v>1</x:v>
@@ -11035,7 +11035,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="I366" s="0">
-        <x:v>0</x:v>
+        <x:v>1E-06</x:v>
       </x:c>
       <x:c r="W366" s="0">
         <x:v>1</x:v>
@@ -11058,7 +11058,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="I367" s="0">
-        <x:v>32.41</x:v>
+        <x:v>1E-06</x:v>
       </x:c>
       <x:c r="W367" s="0">
         <x:v>1</x:v>
@@ -11081,7 +11081,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="I368" s="0">
-        <x:v>0</x:v>
+        <x:v>1E-06</x:v>
       </x:c>
       <x:c r="W368" s="0">
         <x:v>1</x:v>
@@ -11104,7 +11104,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="I369" s="0">
-        <x:v>0.02</x:v>
+        <x:v>1E-06</x:v>
       </x:c>
       <x:c r="W369" s="0">
         <x:v>1</x:v>
@@ -11127,7 +11127,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="I370" s="0">
-        <x:v>0.02</x:v>
+        <x:v>1E-06</x:v>
       </x:c>
       <x:c r="W370" s="0">
         <x:v>1</x:v>
@@ -11150,7 +11150,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="I371" s="0">
-        <x:v>2.25</x:v>
+        <x:v>1E-06</x:v>
       </x:c>
       <x:c r="W371" s="0">
         <x:v>1</x:v>
@@ -11173,7 +11173,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="I372" s="0">
-        <x:v>0.02</x:v>
+        <x:v>1E-06</x:v>
       </x:c>
       <x:c r="W372" s="0">
         <x:v>1</x:v>
@@ -11196,7 +11196,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="I373" s="0">
-        <x:v>0.02</x:v>
+        <x:v>1E-06</x:v>
       </x:c>
       <x:c r="W373" s="0">
         <x:v>1</x:v>
@@ -11219,7 +11219,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="I374" s="0">
-        <x:v>0.02</x:v>
+        <x:v>1E-06</x:v>
       </x:c>
       <x:c r="W374" s="0">
         <x:v>1</x:v>
@@ -11242,7 +11242,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="I375" s="0">
-        <x:v>0.63</x:v>
+        <x:v>1E-06</x:v>
       </x:c>
       <x:c r="W375" s="0">
         <x:v>1</x:v>
@@ -11265,7 +11265,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="I376" s="0">
-        <x:v>97.98</x:v>
+        <x:v>1E-06</x:v>
       </x:c>
       <x:c r="W376" s="0">
         <x:v>1</x:v>
@@ -11311,7 +11311,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="I378" s="0">
-        <x:v>742.59</x:v>
+        <x:v>1E-06</x:v>
       </x:c>
       <x:c r="W378" s="0">
         <x:v>1</x:v>
@@ -11334,7 +11334,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="I379" s="0">
-        <x:v>0.46</x:v>
+        <x:v>1E-06</x:v>
       </x:c>
       <x:c r="W379" s="0">
         <x:v>1</x:v>
@@ -11357,7 +11357,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="I380" s="0">
-        <x:v>0.02</x:v>
+        <x:v>1E-06</x:v>
       </x:c>
       <x:c r="W380" s="0">
         <x:v>1</x:v>
@@ -11380,7 +11380,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="I381" s="0">
-        <x:v>269</x:v>
+        <x:v>1E-06</x:v>
       </x:c>
       <x:c r="W381" s="0">
         <x:v>1</x:v>
@@ -11403,7 +11403,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="I382" s="0">
-        <x:v>0.02</x:v>
+        <x:v>1E-06</x:v>
       </x:c>
       <x:c r="W382" s="0">
         <x:v>1</x:v>
@@ -11426,7 +11426,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="I383" s="0">
-        <x:v>0</x:v>
+        <x:v>1E-06</x:v>
       </x:c>
       <x:c r="W383" s="0">
         <x:v>1</x:v>
@@ -11449,7 +11449,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="I384" s="0">
-        <x:v>25.32</x:v>
+        <x:v>1E-06</x:v>
       </x:c>
       <x:c r="W384" s="0">
         <x:v>1</x:v>
@@ -11472,7 +11472,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="I385" s="0">
-        <x:v>131.64</x:v>
+        <x:v>1E-06</x:v>
       </x:c>
       <x:c r="W385" s="0">
         <x:v>1</x:v>
@@ -11495,7 +11495,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="I386" s="0">
-        <x:v>371.3</x:v>
+        <x:v>1E-06</x:v>
       </x:c>
       <x:c r="W386" s="0">
         <x:v>1</x:v>
@@ -11518,7 +11518,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="I387" s="0">
-        <x:v>255.27</x:v>
+        <x:v>1E-06</x:v>
       </x:c>
       <x:c r="W387" s="0">
         <x:v>1</x:v>
@@ -11541,7 +11541,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="I388" s="0">
-        <x:v>0.02</x:v>
+        <x:v>1E-06</x:v>
       </x:c>
       <x:c r="W388" s="0">
         <x:v>1</x:v>
@@ -11564,7 +11564,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="I389" s="0">
-        <x:v>13.24</x:v>
+        <x:v>1E-06</x:v>
       </x:c>
       <x:c r="W389" s="0">
         <x:v>1</x:v>
@@ -11587,7 +11587,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="I390" s="0">
-        <x:v>16.03</x:v>
+        <x:v>1E-06</x:v>
       </x:c>
       <x:c r="W390" s="0">
         <x:v>1</x:v>
@@ -11610,7 +11610,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="I391" s="0">
-        <x:v>0.05</x:v>
+        <x:v>1E-06</x:v>
       </x:c>
       <x:c r="W391" s="0">
         <x:v>1</x:v>
@@ -11633,7 +11633,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="I392" s="0">
-        <x:v>1.44</x:v>
+        <x:v>1E-06</x:v>
       </x:c>
       <x:c r="W392" s="0">
         <x:v>1</x:v>
@@ -11656,7 +11656,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="I393" s="0">
-        <x:v>0.02</x:v>
+        <x:v>1E-06</x:v>
       </x:c>
       <x:c r="W393" s="0">
         <x:v>1</x:v>
@@ -11679,7 +11679,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="I394" s="0">
-        <x:v>51.93</x:v>
+        <x:v>1E-06</x:v>
       </x:c>
       <x:c r="W394" s="0">
         <x:v>1</x:v>
@@ -11702,7 +11702,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="I395" s="0">
-        <x:v>13.69</x:v>
+        <x:v>1E-06</x:v>
       </x:c>
       <x:c r="W395" s="0">
         <x:v>1</x:v>
@@ -11725,7 +11725,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="I396" s="0">
-        <x:v>32.88</x:v>
+        <x:v>1E-06</x:v>
       </x:c>
       <x:c r="W396" s="0">
         <x:v>1</x:v>
@@ -11748,7 +11748,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="I397" s="0">
-        <x:v>0</x:v>
+        <x:v>1E-06</x:v>
       </x:c>
       <x:c r="W397" s="0">
         <x:v>1</x:v>
@@ -11771,7 +11771,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="I398" s="0">
-        <x:v>3.69</x:v>
+        <x:v>1E-06</x:v>
       </x:c>
       <x:c r="W398" s="0">
         <x:v>1</x:v>
@@ -11794,7 +11794,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="I399" s="0">
-        <x:v>0</x:v>
+        <x:v>1E-06</x:v>
       </x:c>
       <x:c r="W399" s="0">
         <x:v>1</x:v>
@@ -11817,7 +11817,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="I400" s="0">
-        <x:v>1.73</x:v>
+        <x:v>1E-06</x:v>
       </x:c>
       <x:c r="W400" s="0">
         <x:v>1</x:v>
@@ -11840,7 +11840,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="I401" s="0">
-        <x:v>0</x:v>
+        <x:v>1E-06</x:v>
       </x:c>
       <x:c r="W401" s="0">
         <x:v>1</x:v>
@@ -11863,7 +11863,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="I402" s="0">
-        <x:v>31.75</x:v>
+        <x:v>1E-06</x:v>
       </x:c>
       <x:c r="W402" s="0">
         <x:v>1</x:v>
@@ -11886,7 +11886,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="I403" s="0">
-        <x:v>0</x:v>
+        <x:v>1E-06</x:v>
       </x:c>
       <x:c r="W403" s="0">
         <x:v>1</x:v>
@@ -11909,7 +11909,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="I404" s="0">
-        <x:v>0.02</x:v>
+        <x:v>1E-06</x:v>
       </x:c>
       <x:c r="W404" s="0">
         <x:v>1</x:v>
@@ -11932,7 +11932,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="I405" s="0">
-        <x:v>0.02</x:v>
+        <x:v>1E-06</x:v>
       </x:c>
       <x:c r="W405" s="0">
         <x:v>1</x:v>
@@ -11955,7 +11955,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="I406" s="0">
-        <x:v>2.2</x:v>
+        <x:v>1E-06</x:v>
       </x:c>
       <x:c r="W406" s="0">
         <x:v>1</x:v>
@@ -11978,7 +11978,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="I407" s="0">
-        <x:v>0.02</x:v>
+        <x:v>1E-06</x:v>
       </x:c>
       <x:c r="W407" s="0">
         <x:v>1</x:v>
@@ -12001,7 +12001,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="I408" s="0">
-        <x:v>0.02</x:v>
+        <x:v>1E-06</x:v>
       </x:c>
       <x:c r="W408" s="0">
         <x:v>1</x:v>
@@ -12024,7 +12024,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="I409" s="0">
-        <x:v>0.02</x:v>
+        <x:v>1E-06</x:v>
       </x:c>
       <x:c r="W409" s="0">
         <x:v>1</x:v>
@@ -12047,7 +12047,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="I410" s="0">
-        <x:v>0.62</x:v>
+        <x:v>1E-06</x:v>
       </x:c>
       <x:c r="W410" s="0">
         <x:v>1</x:v>
@@ -12070,7 +12070,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="I411" s="0">
-        <x:v>95.99</x:v>
+        <x:v>1E-06</x:v>
       </x:c>
       <x:c r="W411" s="0">
         <x:v>1</x:v>
@@ -12116,7 +12116,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="I413" s="0">
-        <x:v>1502.21</x:v>
+        <x:v>1E-06</x:v>
       </x:c>
       <x:c r="W413" s="0">
         <x:v>1</x:v>
@@ -12139,7 +12139,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="I414" s="0">
-        <x:v>0.38</x:v>
+        <x:v>1E-06</x:v>
       </x:c>
       <x:c r="W414" s="0">
         <x:v>1</x:v>
@@ -12162,7 +12162,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="I415" s="0">
-        <x:v>0.02</x:v>
+        <x:v>1E-06</x:v>
       </x:c>
       <x:c r="W415" s="0">
         <x:v>1</x:v>
@@ -12185,7 +12185,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="I416" s="0">
-        <x:v>114.84</x:v>
+        <x:v>1E-06</x:v>
       </x:c>
       <x:c r="W416" s="0">
         <x:v>1</x:v>
@@ -12208,7 +12208,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="I417" s="0">
-        <x:v>0.02</x:v>
+        <x:v>1E-06</x:v>
       </x:c>
       <x:c r="W417" s="0">
         <x:v>1</x:v>
@@ -12231,7 +12231,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="I418" s="0">
-        <x:v>0</x:v>
+        <x:v>1E-06</x:v>
       </x:c>
       <x:c r="W418" s="0">
         <x:v>1</x:v>
@@ -12254,7 +12254,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="I419" s="0">
-        <x:v>21.92</x:v>
+        <x:v>1E-06</x:v>
       </x:c>
       <x:c r="W419" s="0">
         <x:v>1</x:v>
@@ -12277,7 +12277,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="I420" s="0">
-        <x:v>128.27</x:v>
+        <x:v>1E-06</x:v>
       </x:c>
       <x:c r="W420" s="0">
         <x:v>1</x:v>
@@ -12300,7 +12300,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="I421" s="0">
-        <x:v>211.24</x:v>
+        <x:v>1E-06</x:v>
       </x:c>
       <x:c r="W421" s="0">
         <x:v>1</x:v>
@@ -12323,7 +12323,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="I422" s="0">
-        <x:v>5.76</x:v>
+        <x:v>1E-06</x:v>
       </x:c>
       <x:c r="W422" s="0">
         <x:v>1</x:v>
@@ -12346,7 +12346,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="I423" s="0">
-        <x:v>11.14</x:v>
+        <x:v>1E-06</x:v>
       </x:c>
       <x:c r="W423" s="0">
         <x:v>1</x:v>
@@ -12369,7 +12369,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="I424" s="0">
-        <x:v>0.04</x:v>
+        <x:v>1E-06</x:v>
       </x:c>
       <x:c r="W424" s="0">
         <x:v>1</x:v>
@@ -12392,7 +12392,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="I425" s="0">
-        <x:v>1.25</x:v>
+        <x:v>1E-06</x:v>
       </x:c>
       <x:c r="W425" s="0">
         <x:v>1</x:v>
@@ -12415,7 +12415,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="I426" s="0">
-        <x:v>0.02</x:v>
+        <x:v>1E-06</x:v>
       </x:c>
       <x:c r="W426" s="0">
         <x:v>1</x:v>
@@ -12438,7 +12438,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="I427" s="0">
-        <x:v>30.34</x:v>
+        <x:v>1E-06</x:v>
       </x:c>
       <x:c r="W427" s="0">
         <x:v>1</x:v>
@@ -12461,7 +12461,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="I428" s="0">
-        <x:v>22.66</x:v>
+        <x:v>1E-06</x:v>
       </x:c>
       <x:c r="W428" s="0">
         <x:v>1</x:v>
@@ -12484,7 +12484,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="I429" s="0">
-        <x:v>18.82</x:v>
+        <x:v>1E-06</x:v>
       </x:c>
       <x:c r="W429" s="0">
         <x:v>1</x:v>
@@ -12507,7 +12507,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="I430" s="0">
-        <x:v>0</x:v>
+        <x:v>1E-06</x:v>
       </x:c>
       <x:c r="W430" s="0">
         <x:v>1</x:v>
@@ -12530,7 +12530,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="I431" s="0">
-        <x:v>3.19</x:v>
+        <x:v>1E-06</x:v>
       </x:c>
       <x:c r="W431" s="0">
         <x:v>1</x:v>
@@ -12553,7 +12553,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="I432" s="0">
-        <x:v>0</x:v>
+        <x:v>1E-06</x:v>
       </x:c>
       <x:c r="W432" s="0">
         <x:v>1</x:v>
@@ -12576,7 +12576,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="I433" s="0">
-        <x:v>1.54</x:v>
+        <x:v>1E-06</x:v>
       </x:c>
       <x:c r="W433" s="0">
         <x:v>1</x:v>
@@ -12599,7 +12599,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="I434" s="0">
-        <x:v>0</x:v>
+        <x:v>1E-06</x:v>
       </x:c>
       <x:c r="W434" s="0">
         <x:v>1</x:v>
@@ -12622,7 +12622,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="I435" s="0">
-        <x:v>30.34</x:v>
+        <x:v>1E-06</x:v>
       </x:c>
       <x:c r="W435" s="0">
         <x:v>1</x:v>
@@ -12645,7 +12645,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="I436" s="0">
-        <x:v>0</x:v>
+        <x:v>1E-06</x:v>
       </x:c>
       <x:c r="W436" s="0">
         <x:v>1</x:v>
@@ -12668,7 +12668,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="I437" s="0">
-        <x:v>0.02</x:v>
+        <x:v>1E-06</x:v>
       </x:c>
       <x:c r="W437" s="0">
         <x:v>1</x:v>
@@ -12691,7 +12691,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="I438" s="0">
-        <x:v>0.02</x:v>
+        <x:v>1E-06</x:v>
       </x:c>
       <x:c r="W438" s="0">
         <x:v>1</x:v>
@@ -12714,7 +12714,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="I439" s="0">
-        <x:v>0.02</x:v>
+        <x:v>1E-06</x:v>
       </x:c>
       <x:c r="W439" s="0">
         <x:v>1</x:v>
@@ -12737,7 +12737,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="I440" s="0">
-        <x:v>1.91</x:v>
+        <x:v>1E-06</x:v>
       </x:c>
       <x:c r="W440" s="0">
         <x:v>1</x:v>
@@ -12760,7 +12760,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="I441" s="0">
-        <x:v>0.02</x:v>
+        <x:v>1E-06</x:v>
       </x:c>
       <x:c r="W441" s="0">
         <x:v>1</x:v>
@@ -12783,7 +12783,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="I442" s="0">
-        <x:v>0.02</x:v>
+        <x:v>1E-06</x:v>
       </x:c>
       <x:c r="W442" s="0">
         <x:v>1</x:v>
@@ -12806,7 +12806,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="I443" s="0">
-        <x:v>0.02</x:v>
+        <x:v>1E-06</x:v>
       </x:c>
       <x:c r="W443" s="0">
         <x:v>1</x:v>
@@ -12829,7 +12829,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="I444" s="0">
-        <x:v>0.02</x:v>
+        <x:v>1E-06</x:v>
       </x:c>
       <x:c r="W444" s="0">
         <x:v>1</x:v>
@@ -12852,7 +12852,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="I445" s="0">
-        <x:v>0.51</x:v>
+        <x:v>1E-06</x:v>
       </x:c>
       <x:c r="W445" s="0">
         <x:v>1</x:v>
@@ -12875,7 +12875,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="I446" s="0">
-        <x:v>79.44</x:v>
+        <x:v>1E-06</x:v>
       </x:c>
       <x:c r="W446" s="0">
         <x:v>1</x:v>
@@ -12921,7 +12921,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="I448" s="0">
-        <x:v>2231.11</x:v>
+        <x:v>1E-06</x:v>
       </x:c>
       <x:c r="W448" s="0">
         <x:v>1</x:v>
@@ -12944,7 +12944,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="I449" s="0">
-        <x:v>0.36</x:v>
+        <x:v>1E-06</x:v>
       </x:c>
       <x:c r="W449" s="0">
         <x:v>1</x:v>
@@ -12967,7 +12967,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="I450" s="0">
-        <x:v>0.02</x:v>
+        <x:v>1E-06</x:v>
       </x:c>
       <x:c r="W450" s="0">
         <x:v>1</x:v>
@@ -12990,7 +12990,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="I451" s="0">
-        <x:v>117.74</x:v>
+        <x:v>1E-06</x:v>
       </x:c>
       <x:c r="W451" s="0">
         <x:v>1</x:v>
@@ -13013,7 +13013,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="I452" s="0">
-        <x:v>0.02</x:v>
+        <x:v>1E-06</x:v>
       </x:c>
       <x:c r="W452" s="0">
         <x:v>1</x:v>
@@ -13036,7 +13036,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="I453" s="0">
-        <x:v>0</x:v>
+        <x:v>1E-06</x:v>
       </x:c>
       <x:c r="W453" s="0">
         <x:v>1</x:v>
@@ -13059,7 +13059,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="I454" s="0">
-        <x:v>20.42</x:v>
+        <x:v>1E-06</x:v>
       </x:c>
       <x:c r="W454" s="0">
         <x:v>1</x:v>
@@ -13082,7 +13082,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="I455" s="0">
-        <x:v>119.52</x:v>
+        <x:v>1E-06</x:v>
       </x:c>
       <x:c r="W455" s="0">
         <x:v>1</x:v>
@@ -13105,7 +13105,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="I456" s="0">
-        <x:v>196.83</x:v>
+        <x:v>1E-06</x:v>
       </x:c>
       <x:c r="W456" s="0">
         <x:v>1</x:v>
@@ -13128,7 +13128,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="I457" s="0">
-        <x:v>5.37</x:v>
+        <x:v>1E-06</x:v>
       </x:c>
       <x:c r="W457" s="0">
         <x:v>1</x:v>
@@ -13151,7 +13151,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="I458" s="0">
-        <x:v>10.38</x:v>
+        <x:v>1E-06</x:v>
       </x:c>
       <x:c r="W458" s="0">
         <x:v>1</x:v>
@@ -13174,7 +13174,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="I459" s="0">
-        <x:v>0.04</x:v>
+        <x:v>1E-06</x:v>
       </x:c>
       <x:c r="W459" s="0">
         <x:v>1</x:v>
@@ -13197,7 +13197,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="I460" s="0">
-        <x:v>1.16</x:v>
+        <x:v>1E-06</x:v>
       </x:c>
       <x:c r="W460" s="0">
         <x:v>1</x:v>
@@ -13220,7 +13220,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="I461" s="0">
-        <x:v>0.02</x:v>
+        <x:v>1E-06</x:v>
       </x:c>
       <x:c r="W461" s="0">
         <x:v>1</x:v>
@@ -13243,7 +13243,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="I462" s="0">
-        <x:v>28.27</x:v>
+        <x:v>1E-06</x:v>
       </x:c>
       <x:c r="W462" s="0">
         <x:v>1</x:v>
@@ -13266,7 +13266,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="I463" s="0">
-        <x:v>21.11</x:v>
+        <x:v>1E-06</x:v>
       </x:c>
       <x:c r="W463" s="0">
         <x:v>1</x:v>
@@ -13289,7 +13289,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="I464" s="0">
-        <x:v>17.54</x:v>
+        <x:v>1E-06</x:v>
       </x:c>
       <x:c r="W464" s="0">
         <x:v>1</x:v>
@@ -13312,7 +13312,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="I465" s="0">
-        <x:v>0</x:v>
+        <x:v>1E-06</x:v>
       </x:c>
       <x:c r="W465" s="0">
         <x:v>1</x:v>
@@ -13335,7 +13335,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="I466" s="0">
-        <x:v>2.97</x:v>
+        <x:v>1E-06</x:v>
       </x:c>
       <x:c r="W466" s="0">
         <x:v>1</x:v>
@@ -13358,7 +13358,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="I467" s="0">
-        <x:v>0</x:v>
+        <x:v>1E-06</x:v>
       </x:c>
       <x:c r="W467" s="0">
         <x:v>1</x:v>
@@ -13381,7 +13381,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="I468" s="0">
-        <x:v>1.43</x:v>
+        <x:v>1E-06</x:v>
       </x:c>
       <x:c r="W468" s="0">
         <x:v>1</x:v>
@@ -13404,7 +13404,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="I469" s="0">
-        <x:v>0</x:v>
+        <x:v>1E-06</x:v>
       </x:c>
       <x:c r="W469" s="0">
         <x:v>1</x:v>
@@ -13427,7 +13427,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="I470" s="0">
-        <x:v>28.27</x:v>
+        <x:v>1E-06</x:v>
       </x:c>
       <x:c r="W470" s="0">
         <x:v>1</x:v>
@@ -13450,7 +13450,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="I471" s="0">
-        <x:v>0</x:v>
+        <x:v>1E-06</x:v>
       </x:c>
       <x:c r="W471" s="0">
         <x:v>1</x:v>
@@ -13473,7 +13473,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="I472" s="0">
-        <x:v>0.02</x:v>
+        <x:v>1E-06</x:v>
       </x:c>
       <x:c r="W472" s="0">
         <x:v>1</x:v>
@@ -13496,7 +13496,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="I473" s="0">
-        <x:v>0.02</x:v>
+        <x:v>1E-06</x:v>
       </x:c>
       <x:c r="W473" s="0">
         <x:v>1</x:v>
@@ -13519,7 +13519,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="I474" s="0">
-        <x:v>0.02</x:v>
+        <x:v>1E-06</x:v>
       </x:c>
       <x:c r="W474" s="0">
         <x:v>1</x:v>
@@ -13542,7 +13542,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="I475" s="0">
-        <x:v>1.78</x:v>
+        <x:v>1E-06</x:v>
       </x:c>
       <x:c r="W475" s="0">
         <x:v>1</x:v>
@@ -13565,7 +13565,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="I476" s="0">
-        <x:v>0.02</x:v>
+        <x:v>1E-06</x:v>
       </x:c>
       <x:c r="W476" s="0">
         <x:v>1</x:v>
@@ -13588,7 +13588,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="I477" s="0">
-        <x:v>0.02</x:v>
+        <x:v>1E-06</x:v>
       </x:c>
       <x:c r="W477" s="0">
         <x:v>1</x:v>
@@ -13611,7 +13611,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="I478" s="0">
-        <x:v>0.02</x:v>
+        <x:v>1E-06</x:v>
       </x:c>
       <x:c r="W478" s="0">
         <x:v>1</x:v>
@@ -13634,7 +13634,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="I479" s="0">
-        <x:v>0.02</x:v>
+        <x:v>1E-06</x:v>
       </x:c>
       <x:c r="W479" s="0">
         <x:v>1</x:v>
@@ -13657,7 +13657,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="I480" s="0">
-        <x:v>0.48</x:v>
+        <x:v>1E-06</x:v>
       </x:c>
       <x:c r="W480" s="0">
         <x:v>1</x:v>
@@ -13680,7 +13680,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="I481" s="0">
-        <x:v>74.02</x:v>
+        <x:v>1E-06</x:v>
       </x:c>
       <x:c r="W481" s="0">
         <x:v>1</x:v>

</xml_diff>